<commit_message>
Add CD 2017-CD3 to B-piece balances and writedown slide
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JyYo2ozkKbuwwKMUKoJFV9
</commit_message>
<xml_diff>
--- a/Conduit_B-Piece_Original_Balances.xlsx
+++ b/Conduit_B-Piece_Original_Balances.xlsx
@@ -161,13 +161,13 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -572,7 +572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L39"/>
+  <dimension ref="B2:L40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -663,20 +663,20 @@
     <row r="6">
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>CCUBS 2017-C1</t>
+          <t>CD 2017-CD3</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>2017-11-30</t>
+          <t>2017-02-14</t>
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>696746122</v>
+        <v>1327484158</v>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>Horizontal</t>
+          <t>L-Shaped (VRR + HRR)</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
@@ -686,11 +686,11 @@
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>D-RR, E-RR, F-RR, G-RR, NR-RR</t>
+          <t>E, F, G</t>
         </is>
       </c>
       <c r="H6" s="9">
-        <f>SUMIFS('Class Detail'!$D$5:$D$120,'Class Detail'!$B$5:$B$120,B6)</f>
+        <f>SUMIFS('Class Detail'!$D$5:$D$123,'Class Detail'!$B$5:$B$123,B6)</f>
         <v/>
       </c>
       <c r="I6" s="10">
@@ -698,7 +698,7 @@
         <v/>
       </c>
       <c r="J6" s="6" t="n">
-        <v>35569494</v>
+        <v>43347451</v>
       </c>
       <c r="K6" s="10">
         <f>IFERROR(J6/H6,0)</f>
@@ -713,16 +713,16 @@
     <row r="7">
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>CGCMT 2017-C4</t>
+          <t>CCUBS 2017-C1</t>
         </is>
       </c>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>2017-10-31</t>
+          <t>2017-11-30</t>
         </is>
       </c>
       <c r="D7" s="14" t="n">
-        <v>977059894</v>
+        <v>696746122</v>
       </c>
       <c r="E7" s="15" t="inlineStr">
         <is>
@@ -736,11 +736,11 @@
       </c>
       <c r="G7" s="15" t="inlineStr">
         <is>
-          <t>E-RR, F-RR, G-RR, H-RR, J-RR</t>
+          <t>D-RR, E-RR, F-RR, G-RR, NR-RR</t>
         </is>
       </c>
       <c r="H7" s="17">
-        <f>SUMIFS('Class Detail'!$D$5:$D$120,'Class Detail'!$B$5:$B$120,B7)</f>
+        <f>SUMIFS('Class Detail'!$D$5:$D$123,'Class Detail'!$B$5:$B$123,B7)</f>
         <v/>
       </c>
       <c r="I7" s="18">
@@ -748,7 +748,7 @@
         <v/>
       </c>
       <c r="J7" s="14" t="n">
-        <v>50142415</v>
+        <v>35569494</v>
       </c>
       <c r="K7" s="18">
         <f>IFERROR(J7/H7,0)</f>
@@ -763,20 +763,20 @@
     <row r="8">
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>DBJPM 2017-C6</t>
+          <t>CGCMT 2017-C4</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>2017-06-29</t>
+          <t>2017-10-31</t>
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>1132400405</v>
+        <v>977059894</v>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>L-Shaped (VRR + HRR)</t>
+          <t>Horizontal</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
@@ -786,11 +786,11 @@
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>E-RR, F-RR, G-RR</t>
+          <t>E-RR, F-RR, G-RR, H-RR, J-RR</t>
         </is>
       </c>
       <c r="H8" s="9">
-        <f>SUMIFS('Class Detail'!$D$5:$D$120,'Class Detail'!$B$5:$B$120,B8)</f>
+        <f>SUMIFS('Class Detail'!$D$5:$D$123,'Class Detail'!$B$5:$B$123,B8)</f>
         <v/>
       </c>
       <c r="I8" s="10">
@@ -798,7 +798,7 @@
         <v/>
       </c>
       <c r="J8" s="6" t="n">
-        <v>28683816</v>
+        <v>50142415</v>
       </c>
       <c r="K8" s="10">
         <f>IFERROR(J8/H8,0)</f>
@@ -813,16 +813,16 @@
     <row r="9">
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>GSMS 2017-GS6</t>
+          <t>DBJPM 2017-C6</t>
         </is>
       </c>
       <c r="C9" s="13" t="inlineStr">
         <is>
-          <t>2017-05-31</t>
+          <t>2017-06-29</t>
         </is>
       </c>
       <c r="D9" s="14" t="n">
-        <v>959131421</v>
+        <v>1132400405</v>
       </c>
       <c r="E9" s="15" t="inlineStr">
         <is>
@@ -836,11 +836,11 @@
       </c>
       <c r="G9" s="15" t="inlineStr">
         <is>
-          <t>E, F, G</t>
+          <t>E-RR, F-RR, G-RR</t>
         </is>
       </c>
       <c r="H9" s="17">
-        <f>SUMIFS('Class Detail'!$D$5:$D$120,'Class Detail'!$B$5:$B$120,B9)</f>
+        <f>SUMIFS('Class Detail'!$D$5:$D$123,'Class Detail'!$B$5:$B$123,B9)</f>
         <v/>
       </c>
       <c r="I9" s="18">
@@ -848,7 +848,7 @@
         <v/>
       </c>
       <c r="J9" s="14" t="n">
-        <v>25197303</v>
+        <v>28683816</v>
       </c>
       <c r="K9" s="18">
         <f>IFERROR(J9/H9,0)</f>
@@ -863,20 +863,20 @@
     <row r="10">
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>GSMS 2017-GS8</t>
+          <t>GSMS 2017-GS6</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>2017-11-30</t>
+          <t>2017-05-31</t>
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>1020392386</v>
+        <v>959131421</v>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>Horizontal</t>
+          <t>L-Shaped (VRR + HRR)</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
@@ -886,11 +886,11 @@
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>E-RR, F-RR, G-RR, H-RR</t>
+          <t>E, F, G</t>
         </is>
       </c>
       <c r="H10" s="9">
-        <f>SUMIFS('Class Detail'!$D$5:$D$120,'Class Detail'!$B$5:$B$120,B10)</f>
+        <f>SUMIFS('Class Detail'!$D$5:$D$123,'Class Detail'!$B$5:$B$123,B10)</f>
         <v/>
       </c>
       <c r="I10" s="10">
@@ -898,7 +898,7 @@
         <v/>
       </c>
       <c r="J10" s="6" t="n">
-        <v>52373515</v>
+        <v>25197303</v>
       </c>
       <c r="K10" s="10">
         <f>IFERROR(J10/H10,0)</f>
@@ -913,20 +913,20 @@
     <row r="11">
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>JPMDB 2017-C7</t>
+          <t>GSMS 2017-GS8</t>
         </is>
       </c>
       <c r="C11" s="13" t="inlineStr">
         <is>
-          <t>2017-10-31</t>
+          <t>2017-11-30</t>
         </is>
       </c>
       <c r="D11" s="14" t="n">
-        <v>1105333296</v>
+        <v>1020392386</v>
       </c>
       <c r="E11" s="15" t="inlineStr">
         <is>
-          <t>L-Shaped (VRR + HRR)</t>
+          <t>Horizontal</t>
         </is>
       </c>
       <c r="F11" s="16" t="inlineStr">
@@ -936,11 +936,11 @@
       </c>
       <c r="G11" s="15" t="inlineStr">
         <is>
-          <t>E-RR, F-RR, G-RR</t>
+          <t>E-RR, F-RR, G-RR, H-RR</t>
         </is>
       </c>
       <c r="H11" s="17">
-        <f>SUMIFS('Class Detail'!$D$5:$D$120,'Class Detail'!$B$5:$B$120,B11)</f>
+        <f>SUMIFS('Class Detail'!$D$5:$D$123,'Class Detail'!$B$5:$B$123,B11)</f>
         <v/>
       </c>
       <c r="I11" s="18">
@@ -948,7 +948,7 @@
         <v/>
       </c>
       <c r="J11" s="14" t="n">
-        <v>26162797</v>
+        <v>52373515</v>
       </c>
       <c r="K11" s="18">
         <f>IFERROR(J11/H11,0)</f>
@@ -963,107 +963,107 @@
     <row r="12">
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>LCCM 2017-LC26</t>
-        </is>
-      </c>
-      <c r="C12" s="20" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="D12" s="21" t="n"/>
-      <c r="E12" s="22" t="inlineStr">
-        <is>
-          <t>Vertical (Ladder, ~2%) + Horizontal (~3% FV)</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>Third party purchaser (not disclosed)</t>
-        </is>
-      </c>
-      <c r="G12" s="22" t="inlineStr">
-        <is>
-          <t>Not public: Rule 144A deal</t>
-        </is>
-      </c>
-      <c r="H12" s="21" t="n"/>
-      <c r="I12" s="10" t="n"/>
-      <c r="J12" s="21" t="n"/>
-      <c r="K12" s="10" t="n"/>
+          <t>JPMDB 2017-C7</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>2017-10-31</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>1105333296</v>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>L-Shaped (VRR + HRR)</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>KKR Real Estate Credit Opportunity Partners</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>E-RR, F-RR, G-RR</t>
+        </is>
+      </c>
+      <c r="H12" s="9">
+        <f>SUMIFS('Class Detail'!$D$5:$D$123,'Class Detail'!$B$5:$B$123,B12)</f>
+        <v/>
+      </c>
+      <c r="I12" s="10">
+        <f>IFERROR(H12/D12,0)</f>
+        <v/>
+      </c>
+      <c r="J12" s="6" t="n">
+        <v>26162797</v>
+      </c>
+      <c r="K12" s="10">
+        <f>IFERROR(J12/H12,0)</f>
+        <v/>
+      </c>
       <c r="L12" s="11" t="inlineStr">
         <is>
-          <t>Ladder 8-K (Aug 2017)</t>
+          <t>Final prospectus (424B2)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>MSBAM 2017-C33</t>
-        </is>
-      </c>
-      <c r="C13" s="13" t="inlineStr">
-        <is>
-          <t>2017-05-12</t>
-        </is>
-      </c>
-      <c r="D13" s="14" t="n">
-        <v>702573982</v>
-      </c>
-      <c r="E13" s="15" t="inlineStr">
-        <is>
-          <t>L-Shaped (VRR + HRR)</t>
-        </is>
-      </c>
-      <c r="F13" s="16" t="inlineStr">
-        <is>
-          <t>KKR Real Estate Credit Opportunity Partners</t>
-        </is>
-      </c>
-      <c r="G13" s="15" t="inlineStr">
-        <is>
-          <t>E, F, G</t>
-        </is>
-      </c>
-      <c r="H13" s="17">
-        <f>SUMIFS('Class Detail'!$D$5:$D$120,'Class Detail'!$B$5:$B$120,B13)</f>
-        <v/>
-      </c>
-      <c r="I13" s="18">
-        <f>IFERROR(H13/D13,0)</f>
-        <v/>
-      </c>
-      <c r="J13" s="14" t="n">
-        <v>19989258</v>
-      </c>
-      <c r="K13" s="18">
-        <f>IFERROR(J13/H13,0)</f>
-        <v/>
-      </c>
+          <t>LCCM 2017-LC26</t>
+        </is>
+      </c>
+      <c r="C13" s="20" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D13" s="21" t="n"/>
+      <c r="E13" s="22" t="inlineStr">
+        <is>
+          <t>Vertical (Ladder, ~2%) + Horizontal (~3% FV)</t>
+        </is>
+      </c>
+      <c r="F13" s="12" t="inlineStr">
+        <is>
+          <t>Third party purchaser (not disclosed)</t>
+        </is>
+      </c>
+      <c r="G13" s="22" t="inlineStr">
+        <is>
+          <t>Not public: Rule 144A deal</t>
+        </is>
+      </c>
+      <c r="H13" s="21" t="n"/>
+      <c r="I13" s="18" t="n"/>
+      <c r="J13" s="21" t="n"/>
+      <c r="K13" s="18" t="n"/>
       <c r="L13" s="19" t="inlineStr">
         <is>
-          <t>Final prospectus (424B2)</t>
+          <t>Ladder 8-K (Aug 2017)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>UBSCM 2017-C2</t>
+          <t>MSBAM 2017-C33</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>2017-08-17</t>
+          <t>2017-05-12</t>
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>898681592</v>
+        <v>702573982</v>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>Horizontal</t>
+          <t>L-Shaped (VRR + HRR)</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
@@ -1073,11 +1073,11 @@
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>D-RR, E-RR, F-RR, G-RR, H-RR, NR-RR</t>
+          <t>E, F, G</t>
         </is>
       </c>
       <c r="H14" s="9">
-        <f>SUMIFS('Class Detail'!$D$5:$D$120,'Class Detail'!$B$5:$B$120,B14)</f>
+        <f>SUMIFS('Class Detail'!$D$5:$D$123,'Class Detail'!$B$5:$B$123,B14)</f>
         <v/>
       </c>
       <c r="I14" s="10">
@@ -1085,7 +1085,7 @@
         <v/>
       </c>
       <c r="J14" s="6" t="n">
-        <v>46811027</v>
+        <v>19989258</v>
       </c>
       <c r="K14" s="10">
         <f>IFERROR(J14/H14,0)</f>
@@ -1100,16 +1100,16 @@
     <row r="15">
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>UBSCM 2017-C3</t>
+          <t>UBSCM 2017-C2</t>
         </is>
       </c>
       <c r="C15" s="13" t="inlineStr">
         <is>
-          <t>2017-08-31</t>
+          <t>2017-08-17</t>
         </is>
       </c>
       <c r="D15" s="14" t="n">
-        <v>708626196</v>
+        <v>898681592</v>
       </c>
       <c r="E15" s="15" t="inlineStr">
         <is>
@@ -1123,11 +1123,11 @@
       </c>
       <c r="G15" s="15" t="inlineStr">
         <is>
-          <t>D-RR, E-RR, F-RR, G-RR, NR-RR</t>
+          <t>D-RR, E-RR, F-RR, G-RR, H-RR, NR-RR</t>
         </is>
       </c>
       <c r="H15" s="17">
-        <f>SUMIFS('Class Detail'!$D$5:$D$120,'Class Detail'!$B$5:$B$120,B15)</f>
+        <f>SUMIFS('Class Detail'!$D$5:$D$123,'Class Detail'!$B$5:$B$123,B15)</f>
         <v/>
       </c>
       <c r="I15" s="18">
@@ -1135,7 +1135,7 @@
         <v/>
       </c>
       <c r="J15" s="14" t="n">
-        <v>38157487</v>
+        <v>46811027</v>
       </c>
       <c r="K15" s="18">
         <f>IFERROR(J15/H15,0)</f>
@@ -1150,16 +1150,16 @@
     <row r="16">
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>UBSCM 2017-C5</t>
+          <t>UBSCM 2017-C3</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>2017-11-16</t>
+          <t>2017-08-31</t>
         </is>
       </c>
       <c r="D16" s="6" t="n">
-        <v>743403651</v>
+        <v>708626196</v>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
@@ -1177,7 +1177,7 @@
         </is>
       </c>
       <c r="H16" s="9">
-        <f>SUMIFS('Class Detail'!$D$5:$D$120,'Class Detail'!$B$5:$B$120,B16)</f>
+        <f>SUMIFS('Class Detail'!$D$5:$D$123,'Class Detail'!$B$5:$B$123,B16)</f>
         <v/>
       </c>
       <c r="I16" s="10">
@@ -1185,7 +1185,7 @@
         <v/>
       </c>
       <c r="J16" s="6" t="n">
-        <v>38300901</v>
+        <v>38157487</v>
       </c>
       <c r="K16" s="10">
         <f>IFERROR(J16/H16,0)</f>
@@ -1200,16 +1200,16 @@
     <row r="17">
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>BMARK 2018-B3</t>
+          <t>UBSCM 2017-C5</t>
         </is>
       </c>
       <c r="C17" s="13" t="inlineStr">
         <is>
-          <t>2018-04-10</t>
+          <t>2017-11-16</t>
         </is>
       </c>
       <c r="D17" s="14" t="n">
-        <v>1092537712</v>
+        <v>743403651</v>
       </c>
       <c r="E17" s="15" t="inlineStr">
         <is>
@@ -1223,11 +1223,11 @@
       </c>
       <c r="G17" s="15" t="inlineStr">
         <is>
-          <t>E-RR, F-RR, G-RR, H-RR, NR-RR</t>
+          <t>D-RR, E-RR, F-RR, G-RR, NR-RR</t>
         </is>
       </c>
       <c r="H17" s="17">
-        <f>SUMIFS('Class Detail'!$D$5:$D$120,'Class Detail'!$B$5:$B$120,B17)</f>
+        <f>SUMIFS('Class Detail'!$D$5:$D$123,'Class Detail'!$B$5:$B$123,B17)</f>
         <v/>
       </c>
       <c r="I17" s="18">
@@ -1235,7 +1235,7 @@
         <v/>
       </c>
       <c r="J17" s="14" t="n">
-        <v>55125852</v>
+        <v>38300901</v>
       </c>
       <c r="K17" s="18">
         <f>IFERROR(J17/H17,0)</f>
@@ -1250,20 +1250,20 @@
     <row r="18">
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>BMARK 2018-B6</t>
+          <t>BMARK 2018-B3</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>2018-10-09</t>
+          <t>2018-04-10</t>
         </is>
       </c>
       <c r="D18" s="6" t="n">
-        <v>1147029582</v>
+        <v>1092537712</v>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>L-Shaped (VRR + HRR)</t>
+          <t>Horizontal</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
@@ -1273,11 +1273,11 @@
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>F-RR, G-RR, J-RR, NR-RR</t>
+          <t>E-RR, F-RR, G-RR, H-RR, NR-RR</t>
         </is>
       </c>
       <c r="H18" s="9">
-        <f>SUMIFS('Class Detail'!$D$5:$D$120,'Class Detail'!$B$5:$B$120,B18)</f>
+        <f>SUMIFS('Class Detail'!$D$5:$D$123,'Class Detail'!$B$5:$B$123,B18)</f>
         <v/>
       </c>
       <c r="I18" s="10">
@@ -1285,7 +1285,7 @@
         <v/>
       </c>
       <c r="J18" s="6" t="n">
-        <v>28797132</v>
+        <v>55125852</v>
       </c>
       <c r="K18" s="10">
         <f>IFERROR(J18/H18,0)</f>
@@ -1300,20 +1300,20 @@
     <row r="19">
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>CGCMT 2018-C6</t>
+          <t>BMARK 2018-B6</t>
         </is>
       </c>
       <c r="C19" s="13" t="inlineStr">
         <is>
-          <t>2018-12-11</t>
+          <t>2018-10-09</t>
         </is>
       </c>
       <c r="D19" s="14" t="n">
-        <v>736399174</v>
+        <v>1147029582</v>
       </c>
       <c r="E19" s="15" t="inlineStr">
         <is>
-          <t>Horizontal</t>
+          <t>L-Shaped (VRR + HRR)</t>
         </is>
       </c>
       <c r="F19" s="16" t="inlineStr">
@@ -1323,11 +1323,11 @@
       </c>
       <c r="G19" s="15" t="inlineStr">
         <is>
-          <t>E-RR, F-RR, G-RR, J-RR, K-RR, NR-RR</t>
+          <t>F-RR, G-RR, J-RR, NR-RR</t>
         </is>
       </c>
       <c r="H19" s="17">
-        <f>SUMIFS('Class Detail'!$D$5:$D$120,'Class Detail'!$B$5:$B$120,B19)</f>
+        <f>SUMIFS('Class Detail'!$D$5:$D$123,'Class Detail'!$B$5:$B$123,B19)</f>
         <v/>
       </c>
       <c r="I19" s="18">
@@ -1335,7 +1335,7 @@
         <v/>
       </c>
       <c r="J19" s="14" t="n">
-        <v>38590822</v>
+        <v>28797132</v>
       </c>
       <c r="K19" s="18">
         <f>IFERROR(J19/H19,0)</f>
@@ -1350,20 +1350,20 @@
     <row r="20">
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>MSC 2018-L1</t>
+          <t>CGCMT 2018-C6</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>2018-10-23</t>
+          <t>2018-12-11</t>
         </is>
       </c>
       <c r="D20" s="6" t="n">
-        <v>900598709</v>
+        <v>736399174</v>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>L-Shaped (VRR + HRR)</t>
+          <t>Horizontal</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">
@@ -1373,11 +1373,11 @@
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>F-RR, G-RR, H-RR, J-RR</t>
+          <t>E-RR, F-RR, G-RR, J-RR, K-RR, NR-RR</t>
         </is>
       </c>
       <c r="H20" s="9">
-        <f>SUMIFS('Class Detail'!$D$5:$D$120,'Class Detail'!$B$5:$B$120,B20)</f>
+        <f>SUMIFS('Class Detail'!$D$5:$D$123,'Class Detail'!$B$5:$B$123,B20)</f>
         <v/>
       </c>
       <c r="I20" s="10">
@@ -1385,7 +1385,7 @@
         <v/>
       </c>
       <c r="J20" s="6" t="n">
-        <v>24782457</v>
+        <v>38590822</v>
       </c>
       <c r="K20" s="10">
         <f>IFERROR(J20/H20,0)</f>
@@ -1400,20 +1400,20 @@
     <row r="21">
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>UBSCM 2018-C12</t>
+          <t>MSC 2018-L1</t>
         </is>
       </c>
       <c r="C21" s="13" t="inlineStr">
         <is>
-          <t>2018-08-28</t>
+          <t>2018-10-23</t>
         </is>
       </c>
       <c r="D21" s="14" t="n">
-        <v>804938824</v>
+        <v>900598709</v>
       </c>
       <c r="E21" s="15" t="inlineStr">
         <is>
-          <t>Horizontal</t>
+          <t>L-Shaped (VRR + HRR)</t>
         </is>
       </c>
       <c r="F21" s="16" t="inlineStr">
@@ -1423,11 +1423,11 @@
       </c>
       <c r="G21" s="15" t="inlineStr">
         <is>
-          <t>D-RR, E-RR, F-RR, G-RR, NR-RR</t>
+          <t>F-RR, G-RR, H-RR, J-RR</t>
         </is>
       </c>
       <c r="H21" s="17">
-        <f>SUMIFS('Class Detail'!$D$5:$D$120,'Class Detail'!$B$5:$B$120,B21)</f>
+        <f>SUMIFS('Class Detail'!$D$5:$D$123,'Class Detail'!$B$5:$B$123,B21)</f>
         <v/>
       </c>
       <c r="I21" s="18">
@@ -1435,7 +1435,7 @@
         <v/>
       </c>
       <c r="J21" s="14" t="n">
-        <v>41157452</v>
+        <v>24782457</v>
       </c>
       <c r="K21" s="18">
         <f>IFERROR(J21/H21,0)</f>
@@ -1450,16 +1450,16 @@
     <row r="22">
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>UBSCM 2018-C13</t>
+          <t>UBSCM 2018-C12</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>2018-10-11</t>
+          <t>2018-08-28</t>
         </is>
       </c>
       <c r="D22" s="6" t="n">
-        <v>714880368</v>
+        <v>804938824</v>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
@@ -1477,7 +1477,7 @@
         </is>
       </c>
       <c r="H22" s="9">
-        <f>SUMIFS('Class Detail'!$D$5:$D$120,'Class Detail'!$B$5:$B$120,B22)</f>
+        <f>SUMIFS('Class Detail'!$D$5:$D$123,'Class Detail'!$B$5:$B$123,B22)</f>
         <v/>
       </c>
       <c r="I22" s="10">
@@ -1485,7 +1485,7 @@
         <v/>
       </c>
       <c r="J22" s="6" t="n">
-        <v>36689696</v>
+        <v>41157452</v>
       </c>
       <c r="K22" s="10">
         <f>IFERROR(J22/H22,0)</f>
@@ -1500,16 +1500,16 @@
     <row r="23">
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>UBSCM 2018-C15</t>
+          <t>UBSCM 2018-C13</t>
         </is>
       </c>
       <c r="C23" s="13" t="inlineStr">
         <is>
-          <t>2018-12-28</t>
+          <t>2018-10-11</t>
         </is>
       </c>
       <c r="D23" s="14" t="n">
-        <v>646477345</v>
+        <v>714880368</v>
       </c>
       <c r="E23" s="15" t="inlineStr">
         <is>
@@ -1527,7 +1527,7 @@
         </is>
       </c>
       <c r="H23" s="17">
-        <f>SUMIFS('Class Detail'!$D$5:$D$120,'Class Detail'!$B$5:$B$120,B23)</f>
+        <f>SUMIFS('Class Detail'!$D$5:$D$123,'Class Detail'!$B$5:$B$123,B23)</f>
         <v/>
       </c>
       <c r="I23" s="18">
@@ -1535,7 +1535,7 @@
         <v/>
       </c>
       <c r="J23" s="14" t="n">
-        <v>33161211</v>
+        <v>36689696</v>
       </c>
       <c r="K23" s="18">
         <f>IFERROR(J23/H23,0)</f>
@@ -1550,16 +1550,16 @@
     <row r="24">
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>UBSCM 2018-C8</t>
+          <t>UBSCM 2018-C15</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>2018-02-27</t>
+          <t>2018-12-28</t>
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>1045167892</v>
+        <v>646477345</v>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
@@ -1573,11 +1573,11 @@
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>D-RR, E-RR, F-RR, NR-RR</t>
+          <t>D-RR, E-RR, F-RR, G-RR, NR-RR</t>
         </is>
       </c>
       <c r="H24" s="9">
-        <f>SUMIFS('Class Detail'!$D$5:$D$120,'Class Detail'!$B$5:$B$120,B24)</f>
+        <f>SUMIFS('Class Detail'!$D$5:$D$123,'Class Detail'!$B$5:$B$123,B24)</f>
         <v/>
       </c>
       <c r="I24" s="10">
@@ -1585,7 +1585,7 @@
         <v/>
       </c>
       <c r="J24" s="6" t="n">
-        <v>53204082</v>
+        <v>33161211</v>
       </c>
       <c r="K24" s="10">
         <f>IFERROR(J24/H24,0)</f>
@@ -1600,20 +1600,20 @@
     <row r="25">
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>WFCM 2018-C43</t>
+          <t>UBSCM 2018-C8</t>
         </is>
       </c>
       <c r="C25" s="13" t="inlineStr">
         <is>
-          <t>2018-03-28</t>
+          <t>2018-02-27</t>
         </is>
       </c>
       <c r="D25" s="14" t="n">
-        <v>722448985</v>
+        <v>1045167892</v>
       </c>
       <c r="E25" s="15" t="inlineStr">
         <is>
-          <t>L-Shaped (VRR + HRR)</t>
+          <t>Horizontal</t>
         </is>
       </c>
       <c r="F25" s="16" t="inlineStr">
@@ -1623,11 +1623,11 @@
       </c>
       <c r="G25" s="15" t="inlineStr">
         <is>
-          <t>E, F, G</t>
+          <t>D-RR, E-RR, F-RR, NR-RR</t>
         </is>
       </c>
       <c r="H25" s="17">
-        <f>SUMIFS('Class Detail'!$D$5:$D$120,'Class Detail'!$B$5:$B$120,B25)</f>
+        <f>SUMIFS('Class Detail'!$D$5:$D$123,'Class Detail'!$B$5:$B$123,B25)</f>
         <v/>
       </c>
       <c r="I25" s="18">
@@ -1635,7 +1635,7 @@
         <v/>
       </c>
       <c r="J25" s="14" t="n">
-        <v>20066514</v>
+        <v>53204082</v>
       </c>
       <c r="K25" s="18">
         <f>IFERROR(J25/H25,0)</f>
@@ -1650,20 +1650,20 @@
     <row r="26">
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>WFCM 2018-C47</t>
+          <t>WFCM 2018-C43</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>2018-10-25</t>
+          <t>2018-03-28</t>
         </is>
       </c>
       <c r="D26" s="6" t="n">
-        <v>951555654</v>
+        <v>722448985</v>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>Horizontal</t>
+          <t>L-Shaped (VRR + HRR)</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">
@@ -1673,11 +1673,11 @@
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>E-RR, F-RR, G-RR, H-RR, J-RR</t>
+          <t>E, F, G</t>
         </is>
       </c>
       <c r="H26" s="9">
-        <f>SUMIFS('Class Detail'!$D$5:$D$120,'Class Detail'!$B$5:$B$120,B26)</f>
+        <f>SUMIFS('Class Detail'!$D$5:$D$123,'Class Detail'!$B$5:$B$123,B26)</f>
         <v/>
       </c>
       <c r="I26" s="10">
@@ -1685,7 +1685,7 @@
         <v/>
       </c>
       <c r="J26" s="6" t="n">
-        <v>48654543</v>
+        <v>20066514</v>
       </c>
       <c r="K26" s="10">
         <f>IFERROR(J26/H26,0)</f>
@@ -1700,16 +1700,16 @@
     <row r="27">
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>BBCMS 2019-C3</t>
+          <t>WFCM 2018-C47</t>
         </is>
       </c>
       <c r="C27" s="13" t="inlineStr">
         <is>
-          <t>2019-06-11</t>
+          <t>2018-10-25</t>
         </is>
       </c>
       <c r="D27" s="14" t="n">
-        <v>936649542</v>
+        <v>951555654</v>
       </c>
       <c r="E27" s="15" t="inlineStr">
         <is>
@@ -1727,7 +1727,7 @@
         </is>
       </c>
       <c r="H27" s="17">
-        <f>SUMIFS('Class Detail'!$D$5:$D$120,'Class Detail'!$B$5:$B$120,B27)</f>
+        <f>SUMIFS('Class Detail'!$D$5:$D$123,'Class Detail'!$B$5:$B$123,B27)</f>
         <v/>
       </c>
       <c r="I27" s="18">
@@ -1735,7 +1735,7 @@
         <v/>
       </c>
       <c r="J27" s="14" t="n">
-        <v>49580194</v>
+        <v>48654543</v>
       </c>
       <c r="K27" s="18">
         <f>IFERROR(J27/H27,0)</f>
@@ -1750,16 +1750,16 @@
     <row r="28">
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>GSMS 2019-GC38</t>
+          <t>BBCMS 2019-C3</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>2019-02-27</t>
+          <t>2019-06-11</t>
         </is>
       </c>
       <c r="D28" s="6" t="n">
-        <v>756444365</v>
+        <v>936649542</v>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
@@ -1773,11 +1773,11 @@
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>E-RR, F-RR, G-RR, H-RR, I-RR</t>
+          <t>E-RR, F-RR, G-RR, H-RR, J-RR</t>
         </is>
       </c>
       <c r="H28" s="9">
-        <f>SUMIFS('Class Detail'!$D$5:$D$120,'Class Detail'!$B$5:$B$120,B28)</f>
+        <f>SUMIFS('Class Detail'!$D$5:$D$123,'Class Detail'!$B$5:$B$123,B28)</f>
         <v/>
       </c>
       <c r="I28" s="10">
@@ -1785,7 +1785,7 @@
         <v/>
       </c>
       <c r="J28" s="6" t="n">
-        <v>39335516</v>
+        <v>49580194</v>
       </c>
       <c r="K28" s="10">
         <f>IFERROR(J28/H28,0)</f>
@@ -1800,16 +1800,16 @@
     <row r="29">
       <c r="B29" s="12" t="inlineStr">
         <is>
-          <t>MSC 2019-H6</t>
+          <t>GSMS 2019-GC38</t>
         </is>
       </c>
       <c r="C29" s="13" t="inlineStr">
         <is>
-          <t>2019-06-19</t>
+          <t>2019-02-27</t>
         </is>
       </c>
       <c r="D29" s="14" t="n">
-        <v>686832759</v>
+        <v>756444365</v>
       </c>
       <c r="E29" s="15" t="inlineStr">
         <is>
@@ -1823,11 +1823,11 @@
       </c>
       <c r="G29" s="15" t="inlineStr">
         <is>
-          <t>E-RR, F-RR, G-RR, H-RR, J-RR, K-RR</t>
+          <t>E-RR, F-RR, G-RR, H-RR, I-RR</t>
         </is>
       </c>
       <c r="H29" s="17">
-        <f>SUMIFS('Class Detail'!$D$5:$D$120,'Class Detail'!$B$5:$B$120,B29)</f>
+        <f>SUMIFS('Class Detail'!$D$5:$D$123,'Class Detail'!$B$5:$B$123,B29)</f>
         <v/>
       </c>
       <c r="I29" s="18">
@@ -1835,7 +1835,7 @@
         <v/>
       </c>
       <c r="J29" s="14" t="n">
-        <v>36246073</v>
+        <v>39335516</v>
       </c>
       <c r="K29" s="18">
         <f>IFERROR(J29/H29,0)</f>
@@ -1850,16 +1850,16 @@
     <row r="30">
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>UBSCM 2019-C16</t>
+          <t>MSC 2019-H6</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>2019-04-16</t>
+          <t>2019-06-19</t>
         </is>
       </c>
       <c r="D30" s="6" t="n">
-        <v>682672051</v>
+        <v>686832759</v>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
@@ -1873,11 +1873,11 @@
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>D-RR, E-RR, F-RR, G-RR, H-RR, NR-RR</t>
+          <t>E-RR, F-RR, G-RR, H-RR, J-RR, K-RR</t>
         </is>
       </c>
       <c r="H30" s="9">
-        <f>SUMIFS('Class Detail'!$D$5:$D$120,'Class Detail'!$B$5:$B$120,B30)</f>
+        <f>SUMIFS('Class Detail'!$D$5:$D$123,'Class Detail'!$B$5:$B$123,B30)</f>
         <v/>
       </c>
       <c r="I30" s="10">
@@ -1885,7 +1885,7 @@
         <v/>
       </c>
       <c r="J30" s="6" t="n">
-        <v>36638887</v>
+        <v>36246073</v>
       </c>
       <c r="K30" s="10">
         <f>IFERROR(J30/H30,0)</f>
@@ -1900,16 +1900,16 @@
     <row r="31">
       <c r="B31" s="12" t="inlineStr">
         <is>
-          <t>WFCM 2019-C49</t>
+          <t>UBSCM 2019-C16</t>
         </is>
       </c>
       <c r="C31" s="13" t="inlineStr">
         <is>
-          <t>2019-03-05</t>
+          <t>2019-04-16</t>
         </is>
       </c>
       <c r="D31" s="14" t="n">
-        <v>774228768</v>
+        <v>682672051</v>
       </c>
       <c r="E31" s="15" t="inlineStr">
         <is>
@@ -1923,11 +1923,11 @@
       </c>
       <c r="G31" s="15" t="inlineStr">
         <is>
-          <t>E-RR, F-RR, G-RR, H-RR, J-RR, K-RR</t>
+          <t>D-RR, E-RR, F-RR, G-RR, H-RR, NR-RR</t>
         </is>
       </c>
       <c r="H31" s="17">
-        <f>SUMIFS('Class Detail'!$D$5:$D$120,'Class Detail'!$B$5:$B$120,B31)</f>
+        <f>SUMIFS('Class Detail'!$D$5:$D$123,'Class Detail'!$B$5:$B$123,B31)</f>
         <v/>
       </c>
       <c r="I31" s="18">
@@ -1935,7 +1935,7 @@
         <v/>
       </c>
       <c r="J31" s="14" t="n">
-        <v>40530203</v>
+        <v>36638887</v>
       </c>
       <c r="K31" s="18">
         <f>IFERROR(J31/H31,0)</f>
@@ -1948,74 +1948,124 @@
       </c>
     </row>
     <row r="32">
-      <c r="B32" s="23" t="inlineStr">
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>WFCM 2019-C49</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>2019-03-05</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="n">
+        <v>774228768</v>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>Horizontal</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>KKR Real Estate Credit Opportunity Partners</t>
+        </is>
+      </c>
+      <c r="G32" s="7" t="inlineStr">
+        <is>
+          <t>E-RR, F-RR, G-RR, H-RR, J-RR, K-RR</t>
+        </is>
+      </c>
+      <c r="H32" s="9">
+        <f>SUMIFS('Class Detail'!$D$5:$D$123,'Class Detail'!$B$5:$B$123,B32)</f>
+        <v/>
+      </c>
+      <c r="I32" s="10">
+        <f>IFERROR(H32/D32,0)</f>
+        <v/>
+      </c>
+      <c r="J32" s="6" t="n">
+        <v>40530203</v>
+      </c>
+      <c r="K32" s="10">
+        <f>IFERROR(J32/H32,0)</f>
+        <v/>
+      </c>
+      <c r="L32" s="11" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="23" t="inlineStr">
         <is>
           <t>Total / Wtd. Avg.</t>
         </is>
       </c>
-      <c r="C32" s="24" t="n"/>
-      <c r="D32" s="25">
-        <f>SUM(D6:D31)</f>
-        <v/>
-      </c>
-      <c r="E32" s="24" t="n"/>
-      <c r="F32" s="24" t="n"/>
-      <c r="G32" s="24" t="n"/>
-      <c r="H32" s="25">
-        <f>SUM(H6:H31)</f>
-        <v/>
-      </c>
-      <c r="I32" s="26">
-        <f>IFERROR(SUMIFS(H6:H31,D6:D31,"&gt;0")/D32,0)</f>
-        <v/>
-      </c>
-      <c r="J32" s="25">
-        <f>SUM(J6:J31)</f>
-        <v/>
-      </c>
-      <c r="K32" s="26">
-        <f>IFERROR(J32/H32,0)</f>
-        <v/>
-      </c>
-      <c r="L32" s="24" t="n"/>
-    </row>
-    <row r="34">
-      <c r="B34" s="27" t="inlineStr">
+      <c r="C33" s="24" t="n"/>
+      <c r="D33" s="25">
+        <f>SUM(D6:D32)</f>
+        <v/>
+      </c>
+      <c r="E33" s="24" t="n"/>
+      <c r="F33" s="24" t="n"/>
+      <c r="G33" s="24" t="n"/>
+      <c r="H33" s="25">
+        <f>SUM(H6:H32)</f>
+        <v/>
+      </c>
+      <c r="I33" s="26">
+        <f>IFERROR(SUMIFS(H6:H32,D6:D32,"&gt;0")/D33,0)</f>
+        <v/>
+      </c>
+      <c r="J33" s="25">
+        <f>SUM(J6:J32)</f>
+        <v/>
+      </c>
+      <c r="K33" s="26">
+        <f>IFERROR(J33/H33,0)</f>
+        <v/>
+      </c>
+      <c r="L33" s="24" t="n"/>
+    </row>
+    <row r="35">
+      <c r="B35" s="27" t="inlineStr">
         <is>
           <t>Notes:</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>Original balances are the initial certificate balances of the HRR classes as stated in each final prospectus; class level detail is on the Class Detail tab.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>In L-shaped deals, the sponsors also retained a vertical (VRR) interest, so the HRR is sized to roughly 2.5% of fair value rather than 5.0%, and HRR balances exclude the VRR interest.</t>
+          <t>Original balances are the initial certificate balances of the HRR classes as stated in each final prospectus; class level detail is on the Class Detail tab.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Purchase price is the aggregate HRR purchase price or fair value at closing disclosed in the prospectus, excluding accrued interest.</t>
+          <t>In L-shaped deals, the sponsors also retained a vertical (VRR) interest, so the HRR is sized to roughly 2.5% of fair value rather than 5.0%, and HRR balances exclude the VRR interest.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>LCCM 2017-LC26 was a Rule 144A transaction not filed on EDGAR; Ladder's 8-K discloses a $625.7M trust with a ~2% retained vertical interest and a ~3% (fair value) horizontal interest sold to a third party purchaser, but no class balances.</t>
+          <t>Purchase price is the aggregate HRR purchase price or fair value at closing disclosed in the prospectus, excluding accrued interest.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>LCCM 2017-LC26 was a Rule 144A transaction not filed on EDGAR; Ladder's 8-K discloses a $625.7M trust with a ~2% retained vertical interest and a ~3% (fair value) horizontal interest sold to a third party purchaser, but no class balances.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>Excludes any non HRR classes (e.g., excess interest or Class S/V/Z certificates) the B-piece buyer may also have received.</t>
         </is>
@@ -2049,6 +2099,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId27"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2060,7 +2111,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E120"/>
+  <dimension ref="B2:E123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -2102,16 +2153,16 @@
     <row r="5">
       <c r="B5" s="28" t="inlineStr">
         <is>
-          <t>CCUBS 2017-C1</t>
+          <t>CD 2017-CD3</t>
         </is>
       </c>
       <c r="C5" s="29" t="inlineStr">
         <is>
-          <t>D-RR</t>
+          <t>E</t>
         </is>
       </c>
       <c r="D5" s="30" t="n">
-        <v>21007000</v>
+        <v>35812000</v>
       </c>
       <c r="E5" s="31" t="inlineStr">
         <is>
@@ -2122,16 +2173,16 @@
     <row r="6">
       <c r="B6" s="28" t="inlineStr">
         <is>
-          <t>CCUBS 2017-C1</t>
+          <t>CD 2017-CD3</t>
         </is>
       </c>
       <c r="C6" s="29" t="inlineStr">
         <is>
-          <t>E-RR</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D6" s="30" t="n">
-        <v>8709000</v>
+        <v>14651000</v>
       </c>
       <c r="E6" s="31" t="inlineStr">
         <is>
@@ -2142,58 +2193,58 @@
     <row r="7">
       <c r="B7" s="28" t="inlineStr">
         <is>
+          <t>CD 2017-CD3</t>
+        </is>
+      </c>
+      <c r="C7" s="29" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="D7" s="30" t="n">
+        <v>60229959</v>
+      </c>
+      <c r="E7" s="31" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="32" t="inlineStr">
+        <is>
           <t>CCUBS 2017-C1</t>
         </is>
       </c>
-      <c r="C7" s="29" t="inlineStr">
-        <is>
-          <t>F-RR</t>
-        </is>
-      </c>
-      <c r="D7" s="30" t="n">
-        <v>7838000</v>
-      </c>
-      <c r="E7" s="31" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" s="28" t="inlineStr">
+      <c r="C8" s="33" t="inlineStr">
+        <is>
+          <t>D-RR</t>
+        </is>
+      </c>
+      <c r="D8" s="34" t="n">
+        <v>21007000</v>
+      </c>
+      <c r="E8" s="35" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="32" t="inlineStr">
         <is>
           <t>CCUBS 2017-C1</t>
         </is>
       </c>
-      <c r="C8" s="29" t="inlineStr">
-        <is>
-          <t>G-RR</t>
-        </is>
-      </c>
-      <c r="D8" s="30" t="n">
-        <v>8710000</v>
-      </c>
-      <c r="E8" s="31" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="28" t="inlineStr">
-        <is>
-          <t>CCUBS 2017-C1</t>
-        </is>
-      </c>
-      <c r="C9" s="29" t="inlineStr">
-        <is>
-          <t>NR-RR</t>
-        </is>
-      </c>
-      <c r="D9" s="30" t="n">
-        <v>26128121</v>
-      </c>
-      <c r="E9" s="31" t="inlineStr">
+      <c r="C9" s="33" t="inlineStr">
+        <is>
+          <t>E-RR</t>
+        </is>
+      </c>
+      <c r="D9" s="34" t="n">
+        <v>8709000</v>
+      </c>
+      <c r="E9" s="35" t="inlineStr">
         <is>
           <t>Final prospectus (424B2)</t>
         </is>
@@ -2202,16 +2253,16 @@
     <row r="10">
       <c r="B10" s="32" t="inlineStr">
         <is>
-          <t>CGCMT 2017-C4</t>
+          <t>CCUBS 2017-C1</t>
         </is>
       </c>
       <c r="C10" s="33" t="inlineStr">
         <is>
-          <t>E-RR</t>
+          <t>F-RR</t>
         </is>
       </c>
       <c r="D10" s="34" t="n">
-        <v>21984000</v>
+        <v>7838000</v>
       </c>
       <c r="E10" s="35" t="inlineStr">
         <is>
@@ -2222,16 +2273,16 @@
     <row r="11">
       <c r="B11" s="32" t="inlineStr">
         <is>
-          <t>CGCMT 2017-C4</t>
+          <t>CCUBS 2017-C1</t>
         </is>
       </c>
       <c r="C11" s="33" t="inlineStr">
         <is>
-          <t>F-RR</t>
+          <t>G-RR</t>
         </is>
       </c>
       <c r="D11" s="34" t="n">
-        <v>12214000</v>
+        <v>8710000</v>
       </c>
       <c r="E11" s="35" t="inlineStr">
         <is>
@@ -2242,58 +2293,58 @@
     <row r="12">
       <c r="B12" s="32" t="inlineStr">
         <is>
+          <t>CCUBS 2017-C1</t>
+        </is>
+      </c>
+      <c r="C12" s="33" t="inlineStr">
+        <is>
+          <t>NR-RR</t>
+        </is>
+      </c>
+      <c r="D12" s="34" t="n">
+        <v>26128121</v>
+      </c>
+      <c r="E12" s="35" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="28" t="inlineStr">
+        <is>
           <t>CGCMT 2017-C4</t>
         </is>
       </c>
-      <c r="C12" s="33" t="inlineStr">
-        <is>
-          <t>G-RR</t>
-        </is>
-      </c>
-      <c r="D12" s="34" t="n">
-        <v>12213000</v>
-      </c>
-      <c r="E12" s="35" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="32" t="inlineStr">
+      <c r="C13" s="29" t="inlineStr">
+        <is>
+          <t>E-RR</t>
+        </is>
+      </c>
+      <c r="D13" s="30" t="n">
+        <v>21984000</v>
+      </c>
+      <c r="E13" s="31" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="28" t="inlineStr">
         <is>
           <t>CGCMT 2017-C4</t>
         </is>
       </c>
-      <c r="C13" s="33" t="inlineStr">
-        <is>
-          <t>H-RR</t>
-        </is>
-      </c>
-      <c r="D13" s="34" t="n">
-        <v>9770000</v>
-      </c>
-      <c r="E13" s="35" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="32" t="inlineStr">
-        <is>
-          <t>CGCMT 2017-C4</t>
-        </is>
-      </c>
-      <c r="C14" s="33" t="inlineStr">
-        <is>
-          <t>J-RR</t>
-        </is>
-      </c>
-      <c r="D14" s="34" t="n">
-        <v>48853893</v>
-      </c>
-      <c r="E14" s="35" t="inlineStr">
+      <c r="C14" s="29" t="inlineStr">
+        <is>
+          <t>F-RR</t>
+        </is>
+      </c>
+      <c r="D14" s="30" t="n">
+        <v>12214000</v>
+      </c>
+      <c r="E14" s="31" t="inlineStr">
         <is>
           <t>Final prospectus (424B2)</t>
         </is>
@@ -2302,16 +2353,16 @@
     <row r="15">
       <c r="B15" s="28" t="inlineStr">
         <is>
-          <t>DBJPM 2017-C6</t>
+          <t>CGCMT 2017-C4</t>
         </is>
       </c>
       <c r="C15" s="29" t="inlineStr">
         <is>
-          <t>E-RR</t>
+          <t>G-RR</t>
         </is>
       </c>
       <c r="D15" s="30" t="n">
-        <v>26168000</v>
+        <v>12213000</v>
       </c>
       <c r="E15" s="31" t="inlineStr">
         <is>
@@ -2322,16 +2373,16 @@
     <row r="16">
       <c r="B16" s="28" t="inlineStr">
         <is>
-          <t>DBJPM 2017-C6</t>
+          <t>CGCMT 2017-C4</t>
         </is>
       </c>
       <c r="C16" s="29" t="inlineStr">
         <is>
-          <t>F-RR</t>
+          <t>H-RR</t>
         </is>
       </c>
       <c r="D16" s="30" t="n">
-        <v>11018000</v>
+        <v>9770000</v>
       </c>
       <c r="E16" s="31" t="inlineStr">
         <is>
@@ -2342,16 +2393,16 @@
     <row r="17">
       <c r="B17" s="28" t="inlineStr">
         <is>
-          <t>DBJPM 2017-C6</t>
+          <t>CGCMT 2017-C4</t>
         </is>
       </c>
       <c r="C17" s="29" t="inlineStr">
         <is>
-          <t>G-RR</t>
+          <t>J-RR</t>
         </is>
       </c>
       <c r="D17" s="30" t="n">
-        <v>37187594</v>
+        <v>48853893</v>
       </c>
       <c r="E17" s="31" t="inlineStr">
         <is>
@@ -2362,16 +2413,16 @@
     <row r="18">
       <c r="B18" s="32" t="inlineStr">
         <is>
-          <t>GSMS 2017-GS6</t>
+          <t>DBJPM 2017-C6</t>
         </is>
       </c>
       <c r="C18" s="33" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>E-RR</t>
         </is>
       </c>
       <c r="D18" s="34" t="n">
-        <v>17530000</v>
+        <v>26168000</v>
       </c>
       <c r="E18" s="35" t="inlineStr">
         <is>
@@ -2382,16 +2433,16 @@
     <row r="19">
       <c r="B19" s="32" t="inlineStr">
         <is>
-          <t>GSMS 2017-GS6</t>
+          <t>DBJPM 2017-C6</t>
         </is>
       </c>
       <c r="C19" s="33" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>F-RR</t>
         </is>
       </c>
       <c r="D19" s="34" t="n">
-        <v>10518000</v>
+        <v>11018000</v>
       </c>
       <c r="E19" s="35" t="inlineStr">
         <is>
@@ -2402,16 +2453,16 @@
     <row r="20">
       <c r="B20" s="32" t="inlineStr">
         <is>
-          <t>GSMS 2017-GS6</t>
+          <t>DBJPM 2017-C6</t>
         </is>
       </c>
       <c r="C20" s="33" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>G-RR</t>
         </is>
       </c>
       <c r="D20" s="34" t="n">
-        <v>33893308</v>
+        <v>37187594</v>
       </c>
       <c r="E20" s="35" t="inlineStr">
         <is>
@@ -2422,16 +2473,16 @@
     <row r="21">
       <c r="B21" s="28" t="inlineStr">
         <is>
-          <t>GSMS 2017-GS8</t>
+          <t>GSMS 2017-GS6</t>
         </is>
       </c>
       <c r="C21" s="29" t="inlineStr">
         <is>
-          <t>E-RR</t>
+          <t>E</t>
         </is>
       </c>
       <c r="D21" s="30" t="n">
-        <v>27142000</v>
+        <v>17530000</v>
       </c>
       <c r="E21" s="31" t="inlineStr">
         <is>
@@ -2442,16 +2493,16 @@
     <row r="22">
       <c r="B22" s="28" t="inlineStr">
         <is>
-          <t>GSMS 2017-GS8</t>
+          <t>GSMS 2017-GS6</t>
         </is>
       </c>
       <c r="C22" s="29" t="inlineStr">
         <is>
-          <t>F-RR</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D22" s="30" t="n">
-        <v>26786000</v>
+        <v>10518000</v>
       </c>
       <c r="E22" s="31" t="inlineStr">
         <is>
@@ -2462,38 +2513,38 @@
     <row r="23">
       <c r="B23" s="28" t="inlineStr">
         <is>
+          <t>GSMS 2017-GS6</t>
+        </is>
+      </c>
+      <c r="C23" s="29" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="D23" s="30" t="n">
+        <v>33893308</v>
+      </c>
+      <c r="E23" s="31" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="32" t="inlineStr">
+        <is>
           <t>GSMS 2017-GS8</t>
         </is>
       </c>
-      <c r="C23" s="29" t="inlineStr">
-        <is>
-          <t>G-RR</t>
-        </is>
-      </c>
-      <c r="D23" s="30" t="n">
-        <v>10204000</v>
-      </c>
-      <c r="E23" s="31" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="28" t="inlineStr">
-        <is>
-          <t>GSMS 2017-GS8</t>
-        </is>
-      </c>
-      <c r="C24" s="29" t="inlineStr">
-        <is>
-          <t>H-RR</t>
-        </is>
-      </c>
-      <c r="D24" s="30" t="n">
-        <v>42091386</v>
-      </c>
-      <c r="E24" s="31" t="inlineStr">
+      <c r="C24" s="33" t="inlineStr">
+        <is>
+          <t>E-RR</t>
+        </is>
+      </c>
+      <c r="D24" s="34" t="n">
+        <v>27142000</v>
+      </c>
+      <c r="E24" s="35" t="inlineStr">
         <is>
           <t>Final prospectus (424B2)</t>
         </is>
@@ -2502,16 +2553,16 @@
     <row r="25">
       <c r="B25" s="32" t="inlineStr">
         <is>
-          <t>JPMDB 2017-C7</t>
+          <t>GSMS 2017-GS8</t>
         </is>
       </c>
       <c r="C25" s="33" t="inlineStr">
         <is>
-          <t>E-RR</t>
+          <t>F-RR</t>
         </is>
       </c>
       <c r="D25" s="34" t="n">
-        <v>21499000</v>
+        <v>26786000</v>
       </c>
       <c r="E25" s="35" t="inlineStr">
         <is>
@@ -2522,16 +2573,16 @@
     <row r="26">
       <c r="B26" s="32" t="inlineStr">
         <is>
-          <t>JPMDB 2017-C7</t>
+          <t>GSMS 2017-GS8</t>
         </is>
       </c>
       <c r="C26" s="33" t="inlineStr">
         <is>
-          <t>F-RR</t>
+          <t>G-RR</t>
         </is>
       </c>
       <c r="D26" s="34" t="n">
-        <v>12093000</v>
+        <v>10204000</v>
       </c>
       <c r="E26" s="35" t="inlineStr">
         <is>
@@ -2542,16 +2593,16 @@
     <row r="27">
       <c r="B27" s="32" t="inlineStr">
         <is>
-          <t>JPMDB 2017-C7</t>
+          <t>GSMS 2017-GS8</t>
         </is>
       </c>
       <c r="C27" s="33" t="inlineStr">
         <is>
-          <t>G-RR</t>
+          <t>H-RR</t>
         </is>
       </c>
       <c r="D27" s="34" t="n">
-        <v>36279296</v>
+        <v>42091386</v>
       </c>
       <c r="E27" s="35" t="inlineStr">
         <is>
@@ -2562,16 +2613,16 @@
     <row r="28">
       <c r="B28" s="28" t="inlineStr">
         <is>
-          <t>MSBAM 2017-C33</t>
+          <t>JPMDB 2017-C7</t>
         </is>
       </c>
       <c r="C28" s="29" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>E-RR</t>
         </is>
       </c>
       <c r="D28" s="30" t="n">
-        <v>14564000</v>
+        <v>21499000</v>
       </c>
       <c r="E28" s="31" t="inlineStr">
         <is>
@@ -2582,16 +2633,16 @@
     <row r="29">
       <c r="B29" s="28" t="inlineStr">
         <is>
-          <t>MSBAM 2017-C33</t>
+          <t>JPMDB 2017-C7</t>
         </is>
       </c>
       <c r="C29" s="29" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>F-RR</t>
         </is>
       </c>
       <c r="D29" s="30" t="n">
-        <v>6854000</v>
+        <v>12093000</v>
       </c>
       <c r="E29" s="31" t="inlineStr">
         <is>
@@ -2602,16 +2653,16 @@
     <row r="30">
       <c r="B30" s="28" t="inlineStr">
         <is>
-          <t>MSBAM 2017-C33</t>
+          <t>JPMDB 2017-C7</t>
         </is>
       </c>
       <c r="C30" s="29" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>G-RR</t>
         </is>
       </c>
       <c r="D30" s="30" t="n">
-        <v>26557919</v>
+        <v>36279296</v>
       </c>
       <c r="E30" s="31" t="inlineStr">
         <is>
@@ -2622,16 +2673,16 @@
     <row r="31">
       <c r="B31" s="32" t="inlineStr">
         <is>
-          <t>UBSCM 2017-C2</t>
+          <t>MSBAM 2017-C33</t>
         </is>
       </c>
       <c r="C31" s="33" t="inlineStr">
         <is>
-          <t>D-RR</t>
+          <t>E</t>
         </is>
       </c>
       <c r="D31" s="34" t="n">
-        <v>14514000</v>
+        <v>14564000</v>
       </c>
       <c r="E31" s="35" t="inlineStr">
         <is>
@@ -2642,16 +2693,16 @@
     <row r="32">
       <c r="B32" s="32" t="inlineStr">
         <is>
-          <t>UBSCM 2017-C2</t>
+          <t>MSBAM 2017-C33</t>
         </is>
       </c>
       <c r="C32" s="33" t="inlineStr">
         <is>
-          <t>E-RR</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D32" s="34" t="n">
-        <v>8987000</v>
+        <v>6854000</v>
       </c>
       <c r="E32" s="35" t="inlineStr">
         <is>
@@ -2662,78 +2713,78 @@
     <row r="33">
       <c r="B33" s="32" t="inlineStr">
         <is>
+          <t>MSBAM 2017-C33</t>
+        </is>
+      </c>
+      <c r="C33" s="33" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="D33" s="34" t="n">
+        <v>26557919</v>
+      </c>
+      <c r="E33" s="35" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="28" t="inlineStr">
+        <is>
           <t>UBSCM 2017-C2</t>
         </is>
       </c>
-      <c r="C33" s="33" t="inlineStr">
+      <c r="C34" s="29" t="inlineStr">
+        <is>
+          <t>D-RR</t>
+        </is>
+      </c>
+      <c r="D34" s="30" t="n">
+        <v>14514000</v>
+      </c>
+      <c r="E34" s="31" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="28" t="inlineStr">
+        <is>
+          <t>UBSCM 2017-C2</t>
+        </is>
+      </c>
+      <c r="C35" s="29" t="inlineStr">
+        <is>
+          <t>E-RR</t>
+        </is>
+      </c>
+      <c r="D35" s="30" t="n">
+        <v>8987000</v>
+      </c>
+      <c r="E35" s="31" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="28" t="inlineStr">
+        <is>
+          <t>UBSCM 2017-C2</t>
+        </is>
+      </c>
+      <c r="C36" s="29" t="inlineStr">
         <is>
           <t>F-RR</t>
         </is>
       </c>
-      <c r="D33" s="34" t="n">
+      <c r="D36" s="30" t="n">
         <v>16850000</v>
       </c>
-      <c r="E33" s="35" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="B34" s="32" t="inlineStr">
-        <is>
-          <t>UBSCM 2017-C2</t>
-        </is>
-      </c>
-      <c r="C34" s="33" t="inlineStr">
-        <is>
-          <t>G-RR</t>
-        </is>
-      </c>
-      <c r="D34" s="34" t="n">
-        <v>16850000</v>
-      </c>
-      <c r="E34" s="35" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="B35" s="32" t="inlineStr">
-        <is>
-          <t>UBSCM 2017-C2</t>
-        </is>
-      </c>
-      <c r="C35" s="33" t="inlineStr">
-        <is>
-          <t>H-RR</t>
-        </is>
-      </c>
-      <c r="D35" s="34" t="n">
-        <v>8987000</v>
-      </c>
-      <c r="E35" s="35" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="B36" s="32" t="inlineStr">
-        <is>
-          <t>UBSCM 2017-C2</t>
-        </is>
-      </c>
-      <c r="C36" s="33" t="inlineStr">
-        <is>
-          <t>NR-RR</t>
-        </is>
-      </c>
-      <c r="D36" s="34" t="n">
-        <v>28084591</v>
-      </c>
-      <c r="E36" s="35" t="inlineStr">
+      <c r="E36" s="31" t="inlineStr">
         <is>
           <t>Final prospectus (424B2)</t>
         </is>
@@ -2742,16 +2793,16 @@
     <row r="37">
       <c r="B37" s="28" t="inlineStr">
         <is>
-          <t>UBSCM 2017-C3</t>
+          <t>UBSCM 2017-C2</t>
         </is>
       </c>
       <c r="C37" s="29" t="inlineStr">
         <is>
-          <t>D-RR</t>
+          <t>G-RR</t>
         </is>
       </c>
       <c r="D37" s="30" t="n">
-        <v>17715000</v>
+        <v>16850000</v>
       </c>
       <c r="E37" s="31" t="inlineStr">
         <is>
@@ -2762,16 +2813,16 @@
     <row r="38">
       <c r="B38" s="28" t="inlineStr">
         <is>
-          <t>UBSCM 2017-C3</t>
+          <t>UBSCM 2017-C2</t>
         </is>
       </c>
       <c r="C38" s="29" t="inlineStr">
         <is>
-          <t>E-RR</t>
+          <t>H-RR</t>
         </is>
       </c>
       <c r="D38" s="30" t="n">
-        <v>13287000</v>
+        <v>8987000</v>
       </c>
       <c r="E38" s="31" t="inlineStr">
         <is>
@@ -2782,58 +2833,58 @@
     <row r="39">
       <c r="B39" s="28" t="inlineStr">
         <is>
+          <t>UBSCM 2017-C2</t>
+        </is>
+      </c>
+      <c r="C39" s="29" t="inlineStr">
+        <is>
+          <t>NR-RR</t>
+        </is>
+      </c>
+      <c r="D39" s="30" t="n">
+        <v>28084591</v>
+      </c>
+      <c r="E39" s="31" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="32" t="inlineStr">
+        <is>
           <t>UBSCM 2017-C3</t>
         </is>
       </c>
-      <c r="C39" s="29" t="inlineStr">
-        <is>
-          <t>F-RR</t>
-        </is>
-      </c>
-      <c r="D39" s="30" t="n">
-        <v>10629000</v>
-      </c>
-      <c r="E39" s="31" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="B40" s="28" t="inlineStr">
+      <c r="C40" s="33" t="inlineStr">
+        <is>
+          <t>D-RR</t>
+        </is>
+      </c>
+      <c r="D40" s="34" t="n">
+        <v>17715000</v>
+      </c>
+      <c r="E40" s="35" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="32" t="inlineStr">
         <is>
           <t>UBSCM 2017-C3</t>
         </is>
       </c>
-      <c r="C40" s="29" t="inlineStr">
-        <is>
-          <t>G-RR</t>
-        </is>
-      </c>
-      <c r="D40" s="30" t="n">
-        <v>10630000</v>
-      </c>
-      <c r="E40" s="31" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="B41" s="28" t="inlineStr">
-        <is>
-          <t>UBSCM 2017-C3</t>
-        </is>
-      </c>
-      <c r="C41" s="29" t="inlineStr">
-        <is>
-          <t>NR-RR</t>
-        </is>
-      </c>
-      <c r="D41" s="30" t="n">
-        <v>24802195</v>
-      </c>
-      <c r="E41" s="31" t="inlineStr">
+      <c r="C41" s="33" t="inlineStr">
+        <is>
+          <t>E-RR</t>
+        </is>
+      </c>
+      <c r="D41" s="34" t="n">
+        <v>13287000</v>
+      </c>
+      <c r="E41" s="35" t="inlineStr">
         <is>
           <t>Final prospectus (424B2)</t>
         </is>
@@ -2842,16 +2893,16 @@
     <row r="42">
       <c r="B42" s="32" t="inlineStr">
         <is>
-          <t>UBSCM 2017-C5</t>
+          <t>UBSCM 2017-C3</t>
         </is>
       </c>
       <c r="C42" s="33" t="inlineStr">
         <is>
-          <t>D-RR</t>
+          <t>F-RR</t>
         </is>
       </c>
       <c r="D42" s="34" t="n">
-        <v>15203000</v>
+        <v>10629000</v>
       </c>
       <c r="E42" s="35" t="inlineStr">
         <is>
@@ -2862,16 +2913,16 @@
     <row r="43">
       <c r="B43" s="32" t="inlineStr">
         <is>
-          <t>UBSCM 2017-C5</t>
+          <t>UBSCM 2017-C3</t>
         </is>
       </c>
       <c r="C43" s="33" t="inlineStr">
         <is>
-          <t>E-RR</t>
+          <t>G-RR</t>
         </is>
       </c>
       <c r="D43" s="34" t="n">
-        <v>14868000</v>
+        <v>10630000</v>
       </c>
       <c r="E43" s="35" t="inlineStr">
         <is>
@@ -2882,58 +2933,58 @@
     <row r="44">
       <c r="B44" s="32" t="inlineStr">
         <is>
+          <t>UBSCM 2017-C3</t>
+        </is>
+      </c>
+      <c r="C44" s="33" t="inlineStr">
+        <is>
+          <t>NR-RR</t>
+        </is>
+      </c>
+      <c r="D44" s="34" t="n">
+        <v>24802195</v>
+      </c>
+      <c r="E44" s="35" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="28" t="inlineStr">
+        <is>
           <t>UBSCM 2017-C5</t>
         </is>
       </c>
-      <c r="C44" s="33" t="inlineStr">
-        <is>
-          <t>F-RR</t>
-        </is>
-      </c>
-      <c r="D44" s="34" t="n">
-        <v>15797000</v>
-      </c>
-      <c r="E44" s="35" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="B45" s="32" t="inlineStr">
+      <c r="C45" s="29" t="inlineStr">
+        <is>
+          <t>D-RR</t>
+        </is>
+      </c>
+      <c r="D45" s="30" t="n">
+        <v>15203000</v>
+      </c>
+      <c r="E45" s="31" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="28" t="inlineStr">
         <is>
           <t>UBSCM 2017-C5</t>
         </is>
       </c>
-      <c r="C45" s="33" t="inlineStr">
-        <is>
-          <t>G-RR</t>
-        </is>
-      </c>
-      <c r="D45" s="34" t="n">
-        <v>7434000</v>
-      </c>
-      <c r="E45" s="35" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="B46" s="32" t="inlineStr">
-        <is>
-          <t>UBSCM 2017-C5</t>
-        </is>
-      </c>
-      <c r="C46" s="33" t="inlineStr">
-        <is>
-          <t>NR-RR</t>
-        </is>
-      </c>
-      <c r="D46" s="34" t="n">
-        <v>25090651</v>
-      </c>
-      <c r="E46" s="35" t="inlineStr">
+      <c r="C46" s="29" t="inlineStr">
+        <is>
+          <t>E-RR</t>
+        </is>
+      </c>
+      <c r="D46" s="30" t="n">
+        <v>14868000</v>
+      </c>
+      <c r="E46" s="31" t="inlineStr">
         <is>
           <t>Final prospectus (424B2)</t>
         </is>
@@ -2942,16 +2993,16 @@
     <row r="47">
       <c r="B47" s="28" t="inlineStr">
         <is>
-          <t>BMARK 2018-B3</t>
+          <t>UBSCM 2017-C5</t>
         </is>
       </c>
       <c r="C47" s="29" t="inlineStr">
         <is>
-          <t>E-RR</t>
+          <t>F-RR</t>
         </is>
       </c>
       <c r="D47" s="30" t="n">
-        <v>21924000</v>
+        <v>15797000</v>
       </c>
       <c r="E47" s="31" t="inlineStr">
         <is>
@@ -2962,16 +3013,16 @@
     <row r="48">
       <c r="B48" s="28" t="inlineStr">
         <is>
-          <t>BMARK 2018-B3</t>
+          <t>UBSCM 2017-C5</t>
         </is>
       </c>
       <c r="C48" s="29" t="inlineStr">
         <is>
-          <t>F-RR</t>
+          <t>G-RR</t>
         </is>
       </c>
       <c r="D48" s="30" t="n">
-        <v>12291000</v>
+        <v>7434000</v>
       </c>
       <c r="E48" s="31" t="inlineStr">
         <is>
@@ -2982,58 +3033,58 @@
     <row r="49">
       <c r="B49" s="28" t="inlineStr">
         <is>
+          <t>UBSCM 2017-C5</t>
+        </is>
+      </c>
+      <c r="C49" s="29" t="inlineStr">
+        <is>
+          <t>NR-RR</t>
+        </is>
+      </c>
+      <c r="D49" s="30" t="n">
+        <v>25090651</v>
+      </c>
+      <c r="E49" s="31" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="32" t="inlineStr">
+        <is>
           <t>BMARK 2018-B3</t>
         </is>
       </c>
-      <c r="C49" s="29" t="inlineStr">
-        <is>
-          <t>G-RR</t>
-        </is>
-      </c>
-      <c r="D49" s="30" t="n">
+      <c r="C50" s="33" t="inlineStr">
+        <is>
+          <t>E-RR</t>
+        </is>
+      </c>
+      <c r="D50" s="34" t="n">
+        <v>21924000</v>
+      </c>
+      <c r="E50" s="35" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="32" t="inlineStr">
+        <is>
+          <t>BMARK 2018-B3</t>
+        </is>
+      </c>
+      <c r="C51" s="33" t="inlineStr">
+        <is>
+          <t>F-RR</t>
+        </is>
+      </c>
+      <c r="D51" s="34" t="n">
         <v>12291000</v>
       </c>
-      <c r="E49" s="31" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="B50" s="28" t="inlineStr">
-        <is>
-          <t>BMARK 2018-B3</t>
-        </is>
-      </c>
-      <c r="C50" s="29" t="inlineStr">
-        <is>
-          <t>H-RR</t>
-        </is>
-      </c>
-      <c r="D50" s="30" t="n">
-        <v>15022000</v>
-      </c>
-      <c r="E50" s="31" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="B51" s="28" t="inlineStr">
-        <is>
-          <t>BMARK 2018-B3</t>
-        </is>
-      </c>
-      <c r="C51" s="29" t="inlineStr">
-        <is>
-          <t>NR-RR</t>
-        </is>
-      </c>
-      <c r="D51" s="30" t="n">
-        <v>45067711</v>
-      </c>
-      <c r="E51" s="31" t="inlineStr">
+      <c r="E51" s="35" t="inlineStr">
         <is>
           <t>Final prospectus (424B2)</t>
         </is>
@@ -3042,16 +3093,16 @@
     <row r="52">
       <c r="B52" s="32" t="inlineStr">
         <is>
-          <t>BMARK 2018-B6</t>
+          <t>BMARK 2018-B3</t>
         </is>
       </c>
       <c r="C52" s="33" t="inlineStr">
         <is>
-          <t>F-RR</t>
+          <t>G-RR</t>
         </is>
       </c>
       <c r="D52" s="34" t="n">
-        <v>11175000</v>
+        <v>12291000</v>
       </c>
       <c r="E52" s="35" t="inlineStr">
         <is>
@@ -3062,16 +3113,16 @@
     <row r="53">
       <c r="B53" s="32" t="inlineStr">
         <is>
-          <t>BMARK 2018-B6</t>
+          <t>BMARK 2018-B3</t>
         </is>
       </c>
       <c r="C53" s="33" t="inlineStr">
         <is>
-          <t>G-RR</t>
+          <t>H-RR</t>
         </is>
       </c>
       <c r="D53" s="34" t="n">
-        <v>11176000</v>
+        <v>15022000</v>
       </c>
       <c r="E53" s="35" t="inlineStr">
         <is>
@@ -3082,38 +3133,38 @@
     <row r="54">
       <c r="B54" s="32" t="inlineStr">
         <is>
+          <t>BMARK 2018-B3</t>
+        </is>
+      </c>
+      <c r="C54" s="33" t="inlineStr">
+        <is>
+          <t>NR-RR</t>
+        </is>
+      </c>
+      <c r="D54" s="34" t="n">
+        <v>45067711</v>
+      </c>
+      <c r="E54" s="35" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="28" t="inlineStr">
+        <is>
           <t>BMARK 2018-B6</t>
         </is>
       </c>
-      <c r="C54" s="33" t="inlineStr">
-        <is>
-          <t>J-RR</t>
-        </is>
-      </c>
-      <c r="D54" s="34" t="n">
+      <c r="C55" s="29" t="inlineStr">
+        <is>
+          <t>F-RR</t>
+        </is>
+      </c>
+      <c r="D55" s="30" t="n">
         <v>11175000</v>
       </c>
-      <c r="E54" s="35" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="B55" s="32" t="inlineStr">
-        <is>
-          <t>BMARK 2018-B6</t>
-        </is>
-      </c>
-      <c r="C55" s="33" t="inlineStr">
-        <is>
-          <t>NR-RR</t>
-        </is>
-      </c>
-      <c r="D55" s="34" t="n">
-        <v>33527108</v>
-      </c>
-      <c r="E55" s="35" t="inlineStr">
+      <c r="E55" s="31" t="inlineStr">
         <is>
           <t>Final prospectus (424B2)</t>
         </is>
@@ -3122,16 +3173,16 @@
     <row r="56">
       <c r="B56" s="28" t="inlineStr">
         <is>
-          <t>CGCMT 2018-C6</t>
+          <t>BMARK 2018-B6</t>
         </is>
       </c>
       <c r="C56" s="29" t="inlineStr">
         <is>
-          <t>E-RR</t>
+          <t>G-RR</t>
         </is>
       </c>
       <c r="D56" s="30" t="n">
-        <v>7364000</v>
+        <v>11176000</v>
       </c>
       <c r="E56" s="31" t="inlineStr">
         <is>
@@ -3142,16 +3193,16 @@
     <row r="57">
       <c r="B57" s="28" t="inlineStr">
         <is>
-          <t>CGCMT 2018-C6</t>
+          <t>BMARK 2018-B6</t>
         </is>
       </c>
       <c r="C57" s="29" t="inlineStr">
         <is>
-          <t>F-RR</t>
+          <t>J-RR</t>
         </is>
       </c>
       <c r="D57" s="30" t="n">
-        <v>13807000</v>
+        <v>11175000</v>
       </c>
       <c r="E57" s="31" t="inlineStr">
         <is>
@@ -3162,78 +3213,78 @@
     <row r="58">
       <c r="B58" s="28" t="inlineStr">
         <is>
+          <t>BMARK 2018-B6</t>
+        </is>
+      </c>
+      <c r="C58" s="29" t="inlineStr">
+        <is>
+          <t>NR-RR</t>
+        </is>
+      </c>
+      <c r="D58" s="30" t="n">
+        <v>33527108</v>
+      </c>
+      <c r="E58" s="31" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="32" t="inlineStr">
+        <is>
           <t>CGCMT 2018-C6</t>
         </is>
       </c>
-      <c r="C58" s="29" t="inlineStr">
+      <c r="C59" s="33" t="inlineStr">
+        <is>
+          <t>E-RR</t>
+        </is>
+      </c>
+      <c r="D59" s="34" t="n">
+        <v>7364000</v>
+      </c>
+      <c r="E59" s="35" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="32" t="inlineStr">
+        <is>
+          <t>CGCMT 2018-C6</t>
+        </is>
+      </c>
+      <c r="C60" s="33" t="inlineStr">
+        <is>
+          <t>F-RR</t>
+        </is>
+      </c>
+      <c r="D60" s="34" t="n">
+        <v>13807000</v>
+      </c>
+      <c r="E60" s="35" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="32" t="inlineStr">
+        <is>
+          <t>CGCMT 2018-C6</t>
+        </is>
+      </c>
+      <c r="C61" s="33" t="inlineStr">
         <is>
           <t>G-RR</t>
         </is>
       </c>
-      <c r="D58" s="30" t="n">
+      <c r="D61" s="34" t="n">
         <v>7364000</v>
       </c>
-      <c r="E58" s="31" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="B59" s="28" t="inlineStr">
-        <is>
-          <t>CGCMT 2018-C6</t>
-        </is>
-      </c>
-      <c r="C59" s="29" t="inlineStr">
-        <is>
-          <t>J-RR</t>
-        </is>
-      </c>
-      <c r="D59" s="30" t="n">
-        <v>9205000</v>
-      </c>
-      <c r="E59" s="31" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="B60" s="28" t="inlineStr">
-        <is>
-          <t>CGCMT 2018-C6</t>
-        </is>
-      </c>
-      <c r="C60" s="29" t="inlineStr">
-        <is>
-          <t>K-RR</t>
-        </is>
-      </c>
-      <c r="D60" s="30" t="n">
-        <v>10126000</v>
-      </c>
-      <c r="E60" s="31" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="B61" s="28" t="inlineStr">
-        <is>
-          <t>CGCMT 2018-C6</t>
-        </is>
-      </c>
-      <c r="C61" s="29" t="inlineStr">
-        <is>
-          <t>NR-RR</t>
-        </is>
-      </c>
-      <c r="D61" s="30" t="n">
-        <v>27615173</v>
-      </c>
-      <c r="E61" s="31" t="inlineStr">
+      <c r="E61" s="35" t="inlineStr">
         <is>
           <t>Final prospectus (424B2)</t>
         </is>
@@ -3242,16 +3293,16 @@
     <row r="62">
       <c r="B62" s="32" t="inlineStr">
         <is>
-          <t>MSC 2018-L1</t>
+          <t>CGCMT 2018-C6</t>
         </is>
       </c>
       <c r="C62" s="33" t="inlineStr">
         <is>
-          <t>F-RR</t>
+          <t>J-RR</t>
         </is>
       </c>
       <c r="D62" s="34" t="n">
-        <v>10991000</v>
+        <v>9205000</v>
       </c>
       <c r="E62" s="35" t="inlineStr">
         <is>
@@ -3262,16 +3313,16 @@
     <row r="63">
       <c r="B63" s="32" t="inlineStr">
         <is>
-          <t>MSC 2018-L1</t>
+          <t>CGCMT 2018-C6</t>
         </is>
       </c>
       <c r="C63" s="33" t="inlineStr">
         <is>
-          <t>G-RR</t>
+          <t>K-RR</t>
         </is>
       </c>
       <c r="D63" s="34" t="n">
-        <v>8794000</v>
+        <v>10126000</v>
       </c>
       <c r="E63" s="35" t="inlineStr">
         <is>
@@ -3282,38 +3333,38 @@
     <row r="64">
       <c r="B64" s="32" t="inlineStr">
         <is>
+          <t>CGCMT 2018-C6</t>
+        </is>
+      </c>
+      <c r="C64" s="33" t="inlineStr">
+        <is>
+          <t>NR-RR</t>
+        </is>
+      </c>
+      <c r="D64" s="34" t="n">
+        <v>27615173</v>
+      </c>
+      <c r="E64" s="35" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" s="28" t="inlineStr">
+        <is>
           <t>MSC 2018-L1</t>
         </is>
       </c>
-      <c r="C64" s="33" t="inlineStr">
-        <is>
-          <t>H-RR</t>
-        </is>
-      </c>
-      <c r="D64" s="34" t="n">
-        <v>8793000</v>
-      </c>
-      <c r="E64" s="35" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="B65" s="32" t="inlineStr">
-        <is>
-          <t>MSC 2018-L1</t>
-        </is>
-      </c>
-      <c r="C65" s="33" t="inlineStr">
-        <is>
-          <t>J-RR</t>
-        </is>
-      </c>
-      <c r="D65" s="34" t="n">
-        <v>28579579</v>
-      </c>
-      <c r="E65" s="35" t="inlineStr">
+      <c r="C65" s="29" t="inlineStr">
+        <is>
+          <t>F-RR</t>
+        </is>
+      </c>
+      <c r="D65" s="30" t="n">
+        <v>10991000</v>
+      </c>
+      <c r="E65" s="31" t="inlineStr">
         <is>
           <t>Final prospectus (424B2)</t>
         </is>
@@ -3322,16 +3373,16 @@
     <row r="66">
       <c r="B66" s="28" t="inlineStr">
         <is>
-          <t>UBSCM 2018-C12</t>
+          <t>MSC 2018-L1</t>
         </is>
       </c>
       <c r="C66" s="29" t="inlineStr">
         <is>
-          <t>D-RR</t>
+          <t>G-RR</t>
         </is>
       </c>
       <c r="D66" s="30" t="n">
-        <v>20674000</v>
+        <v>8794000</v>
       </c>
       <c r="E66" s="31" t="inlineStr">
         <is>
@@ -3342,16 +3393,16 @@
     <row r="67">
       <c r="B67" s="28" t="inlineStr">
         <is>
-          <t>UBSCM 2018-C12</t>
+          <t>MSC 2018-L1</t>
         </is>
       </c>
       <c r="C67" s="29" t="inlineStr">
         <is>
-          <t>E-RR</t>
+          <t>H-RR</t>
         </is>
       </c>
       <c r="D67" s="30" t="n">
-        <v>9056000</v>
+        <v>8793000</v>
       </c>
       <c r="E67" s="31" t="inlineStr">
         <is>
@@ -3362,58 +3413,58 @@
     <row r="68">
       <c r="B68" s="28" t="inlineStr">
         <is>
+          <t>MSC 2018-L1</t>
+        </is>
+      </c>
+      <c r="C68" s="29" t="inlineStr">
+        <is>
+          <t>J-RR</t>
+        </is>
+      </c>
+      <c r="D68" s="30" t="n">
+        <v>28579579</v>
+      </c>
+      <c r="E68" s="31" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" s="32" t="inlineStr">
+        <is>
           <t>UBSCM 2018-C12</t>
         </is>
       </c>
-      <c r="C68" s="29" t="inlineStr">
-        <is>
-          <t>F-RR</t>
-        </is>
-      </c>
-      <c r="D68" s="30" t="n">
-        <v>9055000</v>
-      </c>
-      <c r="E68" s="31" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="B69" s="28" t="inlineStr">
+      <c r="C69" s="33" t="inlineStr">
+        <is>
+          <t>D-RR</t>
+        </is>
+      </c>
+      <c r="D69" s="34" t="n">
+        <v>20674000</v>
+      </c>
+      <c r="E69" s="35" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" s="32" t="inlineStr">
         <is>
           <t>UBSCM 2018-C12</t>
         </is>
       </c>
-      <c r="C69" s="29" t="inlineStr">
-        <is>
-          <t>G-RR</t>
-        </is>
-      </c>
-      <c r="D69" s="30" t="n">
+      <c r="C70" s="33" t="inlineStr">
+        <is>
+          <t>E-RR</t>
+        </is>
+      </c>
+      <c r="D70" s="34" t="n">
         <v>9056000</v>
       </c>
-      <c r="E69" s="31" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="B70" s="28" t="inlineStr">
-        <is>
-          <t>UBSCM 2018-C12</t>
-        </is>
-      </c>
-      <c r="C70" s="29" t="inlineStr">
-        <is>
-          <t>NR-RR</t>
-        </is>
-      </c>
-      <c r="D70" s="30" t="n">
-        <v>32197824</v>
-      </c>
-      <c r="E70" s="31" t="inlineStr">
+      <c r="E70" s="35" t="inlineStr">
         <is>
           <t>Final prospectus (424B2)</t>
         </is>
@@ -3422,16 +3473,16 @@
     <row r="71">
       <c r="B71" s="32" t="inlineStr">
         <is>
-          <t>UBSCM 2018-C13</t>
+          <t>UBSCM 2018-C12</t>
         </is>
       </c>
       <c r="C71" s="33" t="inlineStr">
         <is>
-          <t>D-RR</t>
+          <t>F-RR</t>
         </is>
       </c>
       <c r="D71" s="34" t="n">
-        <v>19302000</v>
+        <v>9055000</v>
       </c>
       <c r="E71" s="35" t="inlineStr">
         <is>
@@ -3442,16 +3493,16 @@
     <row r="72">
       <c r="B72" s="32" t="inlineStr">
         <is>
-          <t>UBSCM 2018-C13</t>
+          <t>UBSCM 2018-C12</t>
         </is>
       </c>
       <c r="C72" s="33" t="inlineStr">
         <is>
-          <t>E-RR</t>
+          <t>G-RR</t>
         </is>
       </c>
       <c r="D72" s="34" t="n">
-        <v>8936000</v>
+        <v>9056000</v>
       </c>
       <c r="E72" s="35" t="inlineStr">
         <is>
@@ -3462,58 +3513,58 @@
     <row r="73">
       <c r="B73" s="32" t="inlineStr">
         <is>
+          <t>UBSCM 2018-C12</t>
+        </is>
+      </c>
+      <c r="C73" s="33" t="inlineStr">
+        <is>
+          <t>NR-RR</t>
+        </is>
+      </c>
+      <c r="D73" s="34" t="n">
+        <v>32197824</v>
+      </c>
+      <c r="E73" s="35" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" s="28" t="inlineStr">
+        <is>
           <t>UBSCM 2018-C13</t>
         </is>
       </c>
-      <c r="C73" s="33" t="inlineStr">
-        <is>
-          <t>F-RR</t>
-        </is>
-      </c>
-      <c r="D73" s="34" t="n">
-        <v>7149000</v>
-      </c>
-      <c r="E73" s="35" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="B74" s="32" t="inlineStr">
+      <c r="C74" s="29" t="inlineStr">
+        <is>
+          <t>D-RR</t>
+        </is>
+      </c>
+      <c r="D74" s="30" t="n">
+        <v>19302000</v>
+      </c>
+      <c r="E74" s="31" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" s="28" t="inlineStr">
         <is>
           <t>UBSCM 2018-C13</t>
         </is>
       </c>
-      <c r="C74" s="33" t="inlineStr">
-        <is>
-          <t>G-RR</t>
-        </is>
-      </c>
-      <c r="D74" s="34" t="n">
-        <v>8042000</v>
-      </c>
-      <c r="E74" s="35" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="B75" s="32" t="inlineStr">
-        <is>
-          <t>UBSCM 2018-C13</t>
-        </is>
-      </c>
-      <c r="C75" s="33" t="inlineStr">
-        <is>
-          <t>NR-RR</t>
-        </is>
-      </c>
-      <c r="D75" s="34" t="n">
-        <v>25915367</v>
-      </c>
-      <c r="E75" s="35" t="inlineStr">
+      <c r="C75" s="29" t="inlineStr">
+        <is>
+          <t>E-RR</t>
+        </is>
+      </c>
+      <c r="D75" s="30" t="n">
+        <v>8936000</v>
+      </c>
+      <c r="E75" s="31" t="inlineStr">
         <is>
           <t>Final prospectus (424B2)</t>
         </is>
@@ -3522,16 +3573,16 @@
     <row r="76">
       <c r="B76" s="28" t="inlineStr">
         <is>
-          <t>UBSCM 2018-C15</t>
+          <t>UBSCM 2018-C13</t>
         </is>
       </c>
       <c r="C76" s="29" t="inlineStr">
         <is>
-          <t>D-RR</t>
+          <t>F-RR</t>
         </is>
       </c>
       <c r="D76" s="30" t="n">
-        <v>21444000</v>
+        <v>7149000</v>
       </c>
       <c r="E76" s="31" t="inlineStr">
         <is>
@@ -3542,16 +3593,16 @@
     <row r="77">
       <c r="B77" s="28" t="inlineStr">
         <is>
-          <t>UBSCM 2018-C15</t>
+          <t>UBSCM 2018-C13</t>
         </is>
       </c>
       <c r="C77" s="29" t="inlineStr">
         <is>
-          <t>E-RR</t>
+          <t>G-RR</t>
         </is>
       </c>
       <c r="D77" s="30" t="n">
-        <v>7273000</v>
+        <v>8042000</v>
       </c>
       <c r="E77" s="31" t="inlineStr">
         <is>
@@ -3562,58 +3613,58 @@
     <row r="78">
       <c r="B78" s="28" t="inlineStr">
         <is>
+          <t>UBSCM 2018-C13</t>
+        </is>
+      </c>
+      <c r="C78" s="29" t="inlineStr">
+        <is>
+          <t>NR-RR</t>
+        </is>
+      </c>
+      <c r="D78" s="30" t="n">
+        <v>25915367</v>
+      </c>
+      <c r="E78" s="31" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" s="32" t="inlineStr">
+        <is>
           <t>UBSCM 2018-C15</t>
         </is>
       </c>
-      <c r="C78" s="29" t="inlineStr">
-        <is>
-          <t>F-RR</t>
-        </is>
-      </c>
-      <c r="D78" s="30" t="n">
-        <v>6464000</v>
-      </c>
-      <c r="E78" s="31" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="B79" s="28" t="inlineStr">
+      <c r="C79" s="33" t="inlineStr">
+        <is>
+          <t>D-RR</t>
+        </is>
+      </c>
+      <c r="D79" s="34" t="n">
+        <v>21444000</v>
+      </c>
+      <c r="E79" s="35" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="B80" s="32" t="inlineStr">
         <is>
           <t>UBSCM 2018-C15</t>
         </is>
       </c>
-      <c r="C79" s="29" t="inlineStr">
-        <is>
-          <t>G-RR</t>
-        </is>
-      </c>
-      <c r="D79" s="30" t="n">
-        <v>6465000</v>
-      </c>
-      <c r="E79" s="31" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="B80" s="28" t="inlineStr">
-        <is>
-          <t>UBSCM 2018-C15</t>
-        </is>
-      </c>
-      <c r="C80" s="29" t="inlineStr">
-        <is>
-          <t>NR-RR</t>
-        </is>
-      </c>
-      <c r="D80" s="30" t="n">
-        <v>21819345</v>
-      </c>
-      <c r="E80" s="31" t="inlineStr">
+      <c r="C80" s="33" t="inlineStr">
+        <is>
+          <t>E-RR</t>
+        </is>
+      </c>
+      <c r="D80" s="34" t="n">
+        <v>7273000</v>
+      </c>
+      <c r="E80" s="35" t="inlineStr">
         <is>
           <t>Final prospectus (424B2)</t>
         </is>
@@ -3622,16 +3673,16 @@
     <row r="81">
       <c r="B81" s="32" t="inlineStr">
         <is>
-          <t>UBSCM 2018-C8</t>
+          <t>UBSCM 2018-C15</t>
         </is>
       </c>
       <c r="C81" s="33" t="inlineStr">
         <is>
-          <t>D-RR</t>
+          <t>F-RR</t>
         </is>
       </c>
       <c r="D81" s="34" t="n">
-        <v>31272000</v>
+        <v>6464000</v>
       </c>
       <c r="E81" s="35" t="inlineStr">
         <is>
@@ -3642,16 +3693,16 @@
     <row r="82">
       <c r="B82" s="32" t="inlineStr">
         <is>
-          <t>UBSCM 2018-C8</t>
+          <t>UBSCM 2018-C15</t>
         </is>
       </c>
       <c r="C82" s="33" t="inlineStr">
         <is>
-          <t>E-RR</t>
+          <t>G-RR</t>
         </is>
       </c>
       <c r="D82" s="34" t="n">
-        <v>20903000</v>
+        <v>6465000</v>
       </c>
       <c r="E82" s="35" t="inlineStr">
         <is>
@@ -3662,38 +3713,38 @@
     <row r="83">
       <c r="B83" s="32" t="inlineStr">
         <is>
+          <t>UBSCM 2018-C15</t>
+        </is>
+      </c>
+      <c r="C83" s="33" t="inlineStr">
+        <is>
+          <t>NR-RR</t>
+        </is>
+      </c>
+      <c r="D83" s="34" t="n">
+        <v>21819345</v>
+      </c>
+      <c r="E83" s="35" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="B84" s="28" t="inlineStr">
+        <is>
           <t>UBSCM 2018-C8</t>
         </is>
       </c>
-      <c r="C83" s="33" t="inlineStr">
-        <is>
-          <t>F-RR</t>
-        </is>
-      </c>
-      <c r="D83" s="34" t="n">
-        <v>14371000</v>
-      </c>
-      <c r="E83" s="35" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="B84" s="32" t="inlineStr">
-        <is>
-          <t>UBSCM 2018-C8</t>
-        </is>
-      </c>
-      <c r="C84" s="33" t="inlineStr">
-        <is>
-          <t>NR-RR</t>
-        </is>
-      </c>
-      <c r="D84" s="34" t="n">
-        <v>40500891</v>
-      </c>
-      <c r="E84" s="35" t="inlineStr">
+      <c r="C84" s="29" t="inlineStr">
+        <is>
+          <t>D-RR</t>
+        </is>
+      </c>
+      <c r="D84" s="30" t="n">
+        <v>31272000</v>
+      </c>
+      <c r="E84" s="31" t="inlineStr">
         <is>
           <t>Final prospectus (424B2)</t>
         </is>
@@ -3702,16 +3753,16 @@
     <row r="85">
       <c r="B85" s="28" t="inlineStr">
         <is>
-          <t>WFCM 2018-C43</t>
+          <t>UBSCM 2018-C8</t>
         </is>
       </c>
       <c r="C85" s="29" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>E-RR</t>
         </is>
       </c>
       <c r="D85" s="30" t="n">
-        <v>18519000</v>
+        <v>20903000</v>
       </c>
       <c r="E85" s="31" t="inlineStr">
         <is>
@@ -3722,16 +3773,16 @@
     <row r="86">
       <c r="B86" s="28" t="inlineStr">
         <is>
-          <t>WFCM 2018-C43</t>
+          <t>UBSCM 2018-C8</t>
         </is>
       </c>
       <c r="C86" s="29" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>F-RR</t>
         </is>
       </c>
       <c r="D86" s="30" t="n">
-        <v>8818000</v>
+        <v>14371000</v>
       </c>
       <c r="E86" s="31" t="inlineStr">
         <is>
@@ -3742,16 +3793,16 @@
     <row r="87">
       <c r="B87" s="28" t="inlineStr">
         <is>
-          <t>WFCM 2018-C43</t>
+          <t>UBSCM 2018-C8</t>
         </is>
       </c>
       <c r="C87" s="29" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>NR-RR</t>
         </is>
       </c>
       <c r="D87" s="30" t="n">
-        <v>22046433</v>
+        <v>40500891</v>
       </c>
       <c r="E87" s="31" t="inlineStr">
         <is>
@@ -3762,16 +3813,16 @@
     <row r="88">
       <c r="B88" s="32" t="inlineStr">
         <is>
-          <t>WFCM 2018-C47</t>
+          <t>WFCM 2018-C43</t>
         </is>
       </c>
       <c r="C88" s="33" t="inlineStr">
         <is>
-          <t>E-RR</t>
+          <t>E</t>
         </is>
       </c>
       <c r="D88" s="34" t="n">
-        <v>20501000</v>
+        <v>18519000</v>
       </c>
       <c r="E88" s="35" t="inlineStr">
         <is>
@@ -3782,16 +3833,16 @@
     <row r="89">
       <c r="B89" s="32" t="inlineStr">
         <is>
-          <t>WFCM 2018-C47</t>
+          <t>WFCM 2018-C43</t>
         </is>
       </c>
       <c r="C89" s="33" t="inlineStr">
         <is>
-          <t>F-RR</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D89" s="34" t="n">
-        <v>13084000</v>
+        <v>8818000</v>
       </c>
       <c r="E89" s="35" t="inlineStr">
         <is>
@@ -3802,58 +3853,58 @@
     <row r="90">
       <c r="B90" s="32" t="inlineStr">
         <is>
+          <t>WFCM 2018-C43</t>
+        </is>
+      </c>
+      <c r="C90" s="33" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="D90" s="34" t="n">
+        <v>22046433</v>
+      </c>
+      <c r="E90" s="35" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="B91" s="28" t="inlineStr">
+        <is>
           <t>WFCM 2018-C47</t>
         </is>
       </c>
-      <c r="C90" s="33" t="inlineStr">
-        <is>
-          <t>G-RR</t>
-        </is>
-      </c>
-      <c r="D90" s="34" t="n">
-        <v>10705000</v>
-      </c>
-      <c r="E90" s="35" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="B91" s="32" t="inlineStr">
+      <c r="C91" s="29" t="inlineStr">
+        <is>
+          <t>E-RR</t>
+        </is>
+      </c>
+      <c r="D91" s="30" t="n">
+        <v>20501000</v>
+      </c>
+      <c r="E91" s="31" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="B92" s="28" t="inlineStr">
         <is>
           <t>WFCM 2018-C47</t>
         </is>
       </c>
-      <c r="C91" s="33" t="inlineStr">
-        <is>
-          <t>H-RR</t>
-        </is>
-      </c>
-      <c r="D91" s="34" t="n">
-        <v>9515000</v>
-      </c>
-      <c r="E91" s="35" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="B92" s="32" t="inlineStr">
-        <is>
-          <t>WFCM 2018-C47</t>
-        </is>
-      </c>
-      <c r="C92" s="33" t="inlineStr">
-        <is>
-          <t>J-RR</t>
-        </is>
-      </c>
-      <c r="D92" s="34" t="n">
-        <v>39252654</v>
-      </c>
-      <c r="E92" s="35" t="inlineStr">
+      <c r="C92" s="29" t="inlineStr">
+        <is>
+          <t>F-RR</t>
+        </is>
+      </c>
+      <c r="D92" s="30" t="n">
+        <v>13084000</v>
+      </c>
+      <c r="E92" s="31" t="inlineStr">
         <is>
           <t>Final prospectus (424B2)</t>
         </is>
@@ -3862,16 +3913,16 @@
     <row r="93">
       <c r="B93" s="28" t="inlineStr">
         <is>
-          <t>BBCMS 2019-C3</t>
+          <t>WFCM 2018-C47</t>
         </is>
       </c>
       <c r="C93" s="29" t="inlineStr">
         <is>
-          <t>E-RR</t>
+          <t>G-RR</t>
         </is>
       </c>
       <c r="D93" s="30" t="n">
-        <v>27313000</v>
+        <v>10705000</v>
       </c>
       <c r="E93" s="31" t="inlineStr">
         <is>
@@ -3882,16 +3933,16 @@
     <row r="94">
       <c r="B94" s="28" t="inlineStr">
         <is>
-          <t>BBCMS 2019-C3</t>
+          <t>WFCM 2018-C47</t>
         </is>
       </c>
       <c r="C94" s="29" t="inlineStr">
         <is>
-          <t>F-RR</t>
+          <t>H-RR</t>
         </is>
       </c>
       <c r="D94" s="30" t="n">
-        <v>11708000</v>
+        <v>9515000</v>
       </c>
       <c r="E94" s="31" t="inlineStr">
         <is>
@@ -3902,58 +3953,58 @@
     <row r="95">
       <c r="B95" s="28" t="inlineStr">
         <is>
+          <t>WFCM 2018-C47</t>
+        </is>
+      </c>
+      <c r="C95" s="29" t="inlineStr">
+        <is>
+          <t>J-RR</t>
+        </is>
+      </c>
+      <c r="D95" s="30" t="n">
+        <v>39252654</v>
+      </c>
+      <c r="E95" s="31" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="B96" s="32" t="inlineStr">
+        <is>
           <t>BBCMS 2019-C3</t>
         </is>
       </c>
-      <c r="C95" s="29" t="inlineStr">
-        <is>
-          <t>G-RR</t>
-        </is>
-      </c>
-      <c r="D95" s="30" t="n">
-        <v>10537000</v>
-      </c>
-      <c r="E95" s="31" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="B96" s="28" t="inlineStr">
+      <c r="C96" s="33" t="inlineStr">
+        <is>
+          <t>E-RR</t>
+        </is>
+      </c>
+      <c r="D96" s="34" t="n">
+        <v>27313000</v>
+      </c>
+      <c r="E96" s="35" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="B97" s="32" t="inlineStr">
         <is>
           <t>BBCMS 2019-C3</t>
         </is>
       </c>
-      <c r="C96" s="29" t="inlineStr">
-        <is>
-          <t>H-RR</t>
-        </is>
-      </c>
-      <c r="D96" s="30" t="n">
-        <v>9367000</v>
-      </c>
-      <c r="E96" s="31" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="B97" s="28" t="inlineStr">
-        <is>
-          <t>BBCMS 2019-C3</t>
-        </is>
-      </c>
-      <c r="C97" s="29" t="inlineStr">
-        <is>
-          <t>J-RR</t>
-        </is>
-      </c>
-      <c r="D97" s="30" t="n">
-        <v>36295542</v>
-      </c>
-      <c r="E97" s="31" t="inlineStr">
+      <c r="C97" s="33" t="inlineStr">
+        <is>
+          <t>F-RR</t>
+        </is>
+      </c>
+      <c r="D97" s="34" t="n">
+        <v>11708000</v>
+      </c>
+      <c r="E97" s="35" t="inlineStr">
         <is>
           <t>Final prospectus (424B2)</t>
         </is>
@@ -3962,16 +4013,16 @@
     <row r="98">
       <c r="B98" s="32" t="inlineStr">
         <is>
-          <t>GSMS 2019-GC38</t>
+          <t>BBCMS 2019-C3</t>
         </is>
       </c>
       <c r="C98" s="33" t="inlineStr">
         <is>
-          <t>E-RR</t>
+          <t>G-RR</t>
         </is>
       </c>
       <c r="D98" s="34" t="n">
-        <v>17852000</v>
+        <v>10537000</v>
       </c>
       <c r="E98" s="35" t="inlineStr">
         <is>
@@ -3982,16 +4033,16 @@
     <row r="99">
       <c r="B99" s="32" t="inlineStr">
         <is>
-          <t>GSMS 2019-GC38</t>
+          <t>BBCMS 2019-C3</t>
         </is>
       </c>
       <c r="C99" s="33" t="inlineStr">
         <is>
-          <t>F-RR</t>
+          <t>H-RR</t>
         </is>
       </c>
       <c r="D99" s="34" t="n">
-        <v>9456000</v>
+        <v>9367000</v>
       </c>
       <c r="E99" s="35" t="inlineStr">
         <is>
@@ -4002,58 +4053,58 @@
     <row r="100">
       <c r="B100" s="32" t="inlineStr">
         <is>
+          <t>BBCMS 2019-C3</t>
+        </is>
+      </c>
+      <c r="C100" s="33" t="inlineStr">
+        <is>
+          <t>J-RR</t>
+        </is>
+      </c>
+      <c r="D100" s="34" t="n">
+        <v>36295542</v>
+      </c>
+      <c r="E100" s="35" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="B101" s="28" t="inlineStr">
+        <is>
           <t>GSMS 2019-GC38</t>
         </is>
       </c>
-      <c r="C100" s="33" t="inlineStr">
-        <is>
-          <t>G-RR</t>
-        </is>
-      </c>
-      <c r="D100" s="34" t="n">
-        <v>8510000</v>
-      </c>
-      <c r="E100" s="35" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="B101" s="32" t="inlineStr">
+      <c r="C101" s="29" t="inlineStr">
+        <is>
+          <t>E-RR</t>
+        </is>
+      </c>
+      <c r="D101" s="30" t="n">
+        <v>17852000</v>
+      </c>
+      <c r="E101" s="31" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="B102" s="28" t="inlineStr">
         <is>
           <t>GSMS 2019-GC38</t>
         </is>
       </c>
-      <c r="C101" s="33" t="inlineStr">
-        <is>
-          <t>H-RR</t>
-        </is>
-      </c>
-      <c r="D101" s="34" t="n">
-        <v>7564000</v>
-      </c>
-      <c r="E101" s="35" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="B102" s="32" t="inlineStr">
-        <is>
-          <t>GSMS 2019-GC38</t>
-        </is>
-      </c>
-      <c r="C102" s="33" t="inlineStr">
-        <is>
-          <t>I-RR</t>
-        </is>
-      </c>
-      <c r="D102" s="34" t="n">
-        <v>30258365</v>
-      </c>
-      <c r="E102" s="35" t="inlineStr">
+      <c r="C102" s="29" t="inlineStr">
+        <is>
+          <t>F-RR</t>
+        </is>
+      </c>
+      <c r="D102" s="30" t="n">
+        <v>9456000</v>
+      </c>
+      <c r="E102" s="31" t="inlineStr">
         <is>
           <t>Final prospectus (424B2)</t>
         </is>
@@ -4062,16 +4113,16 @@
     <row r="103">
       <c r="B103" s="28" t="inlineStr">
         <is>
-          <t>MSC 2019-H6</t>
+          <t>GSMS 2019-GC38</t>
         </is>
       </c>
       <c r="C103" s="29" t="inlineStr">
         <is>
-          <t>E-RR</t>
+          <t>G-RR</t>
         </is>
       </c>
       <c r="D103" s="30" t="n">
-        <v>12534000</v>
+        <v>8510000</v>
       </c>
       <c r="E103" s="31" t="inlineStr">
         <is>
@@ -4082,16 +4133,16 @@
     <row r="104">
       <c r="B104" s="28" t="inlineStr">
         <is>
-          <t>MSC 2019-H6</t>
+          <t>GSMS 2019-GC38</t>
         </is>
       </c>
       <c r="C104" s="29" t="inlineStr">
         <is>
-          <t>F-RR</t>
+          <t>H-RR</t>
         </is>
       </c>
       <c r="D104" s="30" t="n">
-        <v>10303000</v>
+        <v>7564000</v>
       </c>
       <c r="E104" s="31" t="inlineStr">
         <is>
@@ -4102,78 +4153,78 @@
     <row r="105">
       <c r="B105" s="28" t="inlineStr">
         <is>
+          <t>GSMS 2019-GC38</t>
+        </is>
+      </c>
+      <c r="C105" s="29" t="inlineStr">
+        <is>
+          <t>I-RR</t>
+        </is>
+      </c>
+      <c r="D105" s="30" t="n">
+        <v>30258365</v>
+      </c>
+      <c r="E105" s="31" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="B106" s="32" t="inlineStr">
+        <is>
           <t>MSC 2019-H6</t>
         </is>
       </c>
-      <c r="C105" s="29" t="inlineStr">
+      <c r="C106" s="33" t="inlineStr">
+        <is>
+          <t>E-RR</t>
+        </is>
+      </c>
+      <c r="D106" s="34" t="n">
+        <v>12534000</v>
+      </c>
+      <c r="E106" s="35" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="B107" s="32" t="inlineStr">
+        <is>
+          <t>MSC 2019-H6</t>
+        </is>
+      </c>
+      <c r="C107" s="33" t="inlineStr">
+        <is>
+          <t>F-RR</t>
+        </is>
+      </c>
+      <c r="D107" s="34" t="n">
+        <v>10303000</v>
+      </c>
+      <c r="E107" s="35" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="B108" s="32" t="inlineStr">
+        <is>
+          <t>MSC 2019-H6</t>
+        </is>
+      </c>
+      <c r="C108" s="33" t="inlineStr">
         <is>
           <t>G-RR</t>
         </is>
       </c>
-      <c r="D105" s="30" t="n">
+      <c r="D108" s="34" t="n">
         <v>7727000</v>
       </c>
-      <c r="E105" s="31" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="B106" s="28" t="inlineStr">
-        <is>
-          <t>MSC 2019-H6</t>
-        </is>
-      </c>
-      <c r="C106" s="29" t="inlineStr">
-        <is>
-          <t>H-RR</t>
-        </is>
-      </c>
-      <c r="D106" s="30" t="n">
-        <v>10302000</v>
-      </c>
-      <c r="E106" s="31" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="B107" s="28" t="inlineStr">
-        <is>
-          <t>MSC 2019-H6</t>
-        </is>
-      </c>
-      <c r="C107" s="29" t="inlineStr">
-        <is>
-          <t>J-RR</t>
-        </is>
-      </c>
-      <c r="D107" s="30" t="n">
-        <v>6869000</v>
-      </c>
-      <c r="E107" s="31" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="B108" s="28" t="inlineStr">
-        <is>
-          <t>MSC 2019-H6</t>
-        </is>
-      </c>
-      <c r="C108" s="29" t="inlineStr">
-        <is>
-          <t>K-RR</t>
-        </is>
-      </c>
-      <c r="D108" s="30" t="n">
-        <v>23180759</v>
-      </c>
-      <c r="E108" s="31" t="inlineStr">
+      <c r="E108" s="35" t="inlineStr">
         <is>
           <t>Final prospectus (424B2)</t>
         </is>
@@ -4182,16 +4233,16 @@
     <row r="109">
       <c r="B109" s="32" t="inlineStr">
         <is>
-          <t>UBSCM 2019-C16</t>
+          <t>MSC 2019-H6</t>
         </is>
       </c>
       <c r="C109" s="33" t="inlineStr">
         <is>
-          <t>D-RR</t>
+          <t>H-RR</t>
         </is>
       </c>
       <c r="D109" s="34" t="n">
-        <v>13695000</v>
+        <v>10302000</v>
       </c>
       <c r="E109" s="35" t="inlineStr">
         <is>
@@ -4202,16 +4253,16 @@
     <row r="110">
       <c r="B110" s="32" t="inlineStr">
         <is>
-          <t>UBSCM 2019-C16</t>
+          <t>MSC 2019-H6</t>
         </is>
       </c>
       <c r="C110" s="33" t="inlineStr">
         <is>
-          <t>E-RR</t>
+          <t>J-RR</t>
         </is>
       </c>
       <c r="D110" s="34" t="n">
-        <v>10240000</v>
+        <v>6869000</v>
       </c>
       <c r="E110" s="35" t="inlineStr">
         <is>
@@ -4222,78 +4273,78 @@
     <row r="111">
       <c r="B111" s="32" t="inlineStr">
         <is>
+          <t>MSC 2019-H6</t>
+        </is>
+      </c>
+      <c r="C111" s="33" t="inlineStr">
+        <is>
+          <t>K-RR</t>
+        </is>
+      </c>
+      <c r="D111" s="34" t="n">
+        <v>23180759</v>
+      </c>
+      <c r="E111" s="35" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="B112" s="28" t="inlineStr">
+        <is>
           <t>UBSCM 2019-C16</t>
         </is>
       </c>
-      <c r="C111" s="33" t="inlineStr">
+      <c r="C112" s="29" t="inlineStr">
+        <is>
+          <t>D-RR</t>
+        </is>
+      </c>
+      <c r="D112" s="30" t="n">
+        <v>13695000</v>
+      </c>
+      <c r="E112" s="31" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="B113" s="28" t="inlineStr">
+        <is>
+          <t>UBSCM 2019-C16</t>
+        </is>
+      </c>
+      <c r="C113" s="29" t="inlineStr">
+        <is>
+          <t>E-RR</t>
+        </is>
+      </c>
+      <c r="D113" s="30" t="n">
+        <v>10240000</v>
+      </c>
+      <c r="E113" s="31" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="B114" s="28" t="inlineStr">
+        <is>
+          <t>UBSCM 2019-C16</t>
+        </is>
+      </c>
+      <c r="C114" s="29" t="inlineStr">
         <is>
           <t>F-RR</t>
         </is>
       </c>
-      <c r="D111" s="34" t="n">
+      <c r="D114" s="30" t="n">
         <v>6827000</v>
       </c>
-      <c r="E111" s="35" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="B112" s="32" t="inlineStr">
-        <is>
-          <t>UBSCM 2019-C16</t>
-        </is>
-      </c>
-      <c r="C112" s="33" t="inlineStr">
-        <is>
-          <t>G-RR</t>
-        </is>
-      </c>
-      <c r="D112" s="34" t="n">
-        <v>8533000</v>
-      </c>
-      <c r="E112" s="35" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="B113" s="32" t="inlineStr">
-        <is>
-          <t>UBSCM 2019-C16</t>
-        </is>
-      </c>
-      <c r="C113" s="33" t="inlineStr">
-        <is>
-          <t>H-RR</t>
-        </is>
-      </c>
-      <c r="D113" s="34" t="n">
-        <v>6827000</v>
-      </c>
-      <c r="E113" s="35" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="B114" s="32" t="inlineStr">
-        <is>
-          <t>UBSCM 2019-C16</t>
-        </is>
-      </c>
-      <c r="C114" s="33" t="inlineStr">
-        <is>
-          <t>NR-RR</t>
-        </is>
-      </c>
-      <c r="D114" s="34" t="n">
-        <v>22187051</v>
-      </c>
-      <c r="E114" s="35" t="inlineStr">
+      <c r="E114" s="31" t="inlineStr">
         <is>
           <t>Final prospectus (424B2)</t>
         </is>
@@ -4302,16 +4353,16 @@
     <row r="115">
       <c r="B115" s="28" t="inlineStr">
         <is>
-          <t>WFCM 2019-C49</t>
+          <t>UBSCM 2019-C16</t>
         </is>
       </c>
       <c r="C115" s="29" t="inlineStr">
         <is>
-          <t>E-RR</t>
+          <t>G-RR</t>
         </is>
       </c>
       <c r="D115" s="30" t="n">
-        <v>18504000</v>
+        <v>8533000</v>
       </c>
       <c r="E115" s="31" t="inlineStr">
         <is>
@@ -4322,16 +4373,16 @@
     <row r="116">
       <c r="B116" s="28" t="inlineStr">
         <is>
-          <t>WFCM 2019-C49</t>
+          <t>UBSCM 2019-C16</t>
         </is>
       </c>
       <c r="C116" s="29" t="inlineStr">
         <is>
-          <t>F-RR</t>
+          <t>H-RR</t>
         </is>
       </c>
       <c r="D116" s="30" t="n">
-        <v>10646000</v>
+        <v>6827000</v>
       </c>
       <c r="E116" s="31" t="inlineStr">
         <is>
@@ -4342,78 +4393,138 @@
     <row r="117">
       <c r="B117" s="28" t="inlineStr">
         <is>
+          <t>UBSCM 2019-C16</t>
+        </is>
+      </c>
+      <c r="C117" s="29" t="inlineStr">
+        <is>
+          <t>NR-RR</t>
+        </is>
+      </c>
+      <c r="D117" s="30" t="n">
+        <v>22187051</v>
+      </c>
+      <c r="E117" s="31" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="B118" s="32" t="inlineStr">
+        <is>
           <t>WFCM 2019-C49</t>
         </is>
       </c>
-      <c r="C117" s="29" t="inlineStr">
+      <c r="C118" s="33" t="inlineStr">
+        <is>
+          <t>E-RR</t>
+        </is>
+      </c>
+      <c r="D118" s="34" t="n">
+        <v>18504000</v>
+      </c>
+      <c r="E118" s="35" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="B119" s="32" t="inlineStr">
+        <is>
+          <t>WFCM 2019-C49</t>
+        </is>
+      </c>
+      <c r="C119" s="33" t="inlineStr">
+        <is>
+          <t>F-RR</t>
+        </is>
+      </c>
+      <c r="D119" s="34" t="n">
+        <v>10646000</v>
+      </c>
+      <c r="E119" s="35" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="B120" s="32" t="inlineStr">
+        <is>
+          <t>WFCM 2019-C49</t>
+        </is>
+      </c>
+      <c r="C120" s="33" t="inlineStr">
         <is>
           <t>G-RR</t>
         </is>
       </c>
-      <c r="D117" s="30" t="n">
+      <c r="D120" s="34" t="n">
         <v>9677000</v>
       </c>
-      <c r="E117" s="31" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="B118" s="28" t="inlineStr">
+      <c r="E120" s="35" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="B121" s="32" t="inlineStr">
         <is>
           <t>WFCM 2019-C49</t>
         </is>
       </c>
-      <c r="C118" s="29" t="inlineStr">
+      <c r="C121" s="33" t="inlineStr">
         <is>
           <t>H-RR</t>
         </is>
       </c>
-      <c r="D118" s="30" t="n">
+      <c r="D121" s="34" t="n">
         <v>8711000</v>
       </c>
-      <c r="E118" s="31" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="B119" s="28" t="inlineStr">
+      <c r="E121" s="35" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="B122" s="32" t="inlineStr">
         <is>
           <t>WFCM 2019-C49</t>
         </is>
       </c>
-      <c r="C119" s="29" t="inlineStr">
+      <c r="C122" s="33" t="inlineStr">
         <is>
           <t>J-RR</t>
         </is>
       </c>
-      <c r="D119" s="30" t="n">
+      <c r="D122" s="34" t="n">
         <v>8710000</v>
       </c>
-      <c r="E119" s="31" t="inlineStr">
-        <is>
-          <t>Final prospectus (424B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="B120" s="28" t="inlineStr">
+      <c r="E122" s="35" t="inlineStr">
+        <is>
+          <t>Final prospectus (424B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="B123" s="32" t="inlineStr">
         <is>
           <t>WFCM 2019-C49</t>
         </is>
       </c>
-      <c r="C120" s="29" t="inlineStr">
+      <c r="C123" s="33" t="inlineStr">
         <is>
           <t>K-RR</t>
         </is>
       </c>
-      <c r="D120" s="30" t="n">
+      <c r="D123" s="34" t="n">
         <v>24194767</v>
       </c>
-      <c r="E120" s="31" t="inlineStr">
+      <c r="E123" s="35" t="inlineStr">
         <is>
           <t>Final prospectus (424B2)</t>
         </is>
@@ -4537,6 +4648,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E118" r:id="rId114"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E119" r:id="rId115"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E120" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E121" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E122" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E123" r:id="rId119"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>